<commit_message>
Populate Ajanta Target Tracker with all 57 purchase bills and 7 settled credit notes
</commit_message>
<xml_diff>
--- a/Ajanta_Target_and_Scheme_Tracker_FY26-27.xlsx
+++ b/Ajanta_Target_and_Scheme_Tracker_FY26-27.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Target Tracker" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly &amp; Annual (QTB-ATB)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inward Bill Quick-Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ajanta Credit Notes Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -150,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -212,6 +213,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -702,8 +710,9 @@
       <c r="C5" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D5" s="5" t="n">
-        <v>1192130.34</v>
+      <c r="D5" s="5">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Aug-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E5" s="6">
         <f>IF(C5&gt;0, D5/C5, 0)</f>
@@ -740,8 +749,9 @@
         <f>K5+L5</f>
         <v/>
       </c>
-      <c r="N5" s="5" t="n">
-        <v>111949.07</v>
+      <c r="N5" s="5">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Aug-2026")</f>
+        <v/>
       </c>
       <c r="O5" s="5">
         <f>M5-N5</f>
@@ -762,8 +772,9 @@
       <c r="C6" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D6" s="9" t="n">
-        <v>997322.76</v>
+      <c r="D6" s="9">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Sep-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E6" s="10">
         <f>IF(C6&gt;0, D6/C6, 0)</f>
@@ -800,8 +811,9 @@
         <f>K6+L6</f>
         <v/>
       </c>
-      <c r="N6" s="9" t="n">
-        <v>86707</v>
+      <c r="N6" s="9">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Sep-2026")</f>
+        <v/>
       </c>
       <c r="O6" s="9">
         <f>M6-N6</f>
@@ -822,8 +834,9 @@
       <c r="C7" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D7" s="5" t="n">
-        <v>0</v>
+      <c r="D7" s="5">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Oct-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E7" s="6">
         <f>IF(C7&gt;0, D7/C7, 0)</f>
@@ -860,8 +873,9 @@
         <f>K7+L7</f>
         <v/>
       </c>
-      <c r="N7" s="5" t="n">
-        <v>0</v>
+      <c r="N7" s="5">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Oct-2026")</f>
+        <v/>
       </c>
       <c r="O7" s="5">
         <f>M7-N7</f>
@@ -882,8 +896,9 @@
       <c r="C8" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>0</v>
+      <c r="D8" s="9">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Nov-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E8" s="10">
         <f>IF(C8&gt;0, D8/C8, 0)</f>
@@ -920,8 +935,9 @@
         <f>K8+L8</f>
         <v/>
       </c>
-      <c r="N8" s="9" t="n">
-        <v>0</v>
+      <c r="N8" s="9">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Nov-2026")</f>
+        <v/>
       </c>
       <c r="O8" s="9">
         <f>M8-N8</f>
@@ -942,8 +958,9 @@
       <c r="C9" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D9" s="5" t="n">
-        <v>0</v>
+      <c r="D9" s="5">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Dec-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E9" s="6">
         <f>IF(C9&gt;0, D9/C9, 0)</f>
@@ -980,8 +997,9 @@
         <f>K9+L9</f>
         <v/>
       </c>
-      <c r="N9" s="5" t="n">
-        <v>0</v>
+      <c r="N9" s="5">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Dec-2026")</f>
+        <v/>
       </c>
       <c r="O9" s="5">
         <f>M9-N9</f>
@@ -1002,8 +1020,9 @@
       <c r="C10" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D10" s="9" t="n">
-        <v>0</v>
+      <c r="D10" s="9">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Jan-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E10" s="10">
         <f>IF(C10&gt;0, D10/C10, 0)</f>
@@ -1040,8 +1059,9 @@
         <f>K10+L10</f>
         <v/>
       </c>
-      <c r="N10" s="9" t="n">
-        <v>0</v>
+      <c r="N10" s="9">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Jan-2027")</f>
+        <v/>
       </c>
       <c r="O10" s="9">
         <f>M10-N10</f>
@@ -1062,8 +1082,9 @@
       <c r="C11" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D11" s="5" t="n">
-        <v>0</v>
+      <c r="D11" s="5">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Feb-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E11" s="6">
         <f>IF(C11&gt;0, D11/C11, 0)</f>
@@ -1100,8 +1121,9 @@
         <f>K11+L11</f>
         <v/>
       </c>
-      <c r="N11" s="5" t="n">
-        <v>0</v>
+      <c r="N11" s="5">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Feb-2027")</f>
+        <v/>
       </c>
       <c r="O11" s="5">
         <f>M11-N11</f>
@@ -1122,8 +1144,9 @@
       <c r="C12" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>0</v>
+      <c r="D12" s="9">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Mar-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E12" s="10">
         <f>IF(C12&gt;0, D12/C12, 0)</f>
@@ -1160,8 +1183,9 @@
         <f>K12+L12</f>
         <v/>
       </c>
-      <c r="N12" s="9" t="n">
-        <v>0</v>
+      <c r="N12" s="9">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Mar-2027")</f>
+        <v/>
       </c>
       <c r="O12" s="9">
         <f>M12-N12</f>
@@ -1182,8 +1206,9 @@
       <c r="C13" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D13" s="5" t="n">
-        <v>0</v>
+      <c r="D13" s="5">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Apr-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E13" s="6">
         <f>IF(C13&gt;0, D13/C13, 0)</f>
@@ -1220,8 +1245,9 @@
         <f>K13+L13</f>
         <v/>
       </c>
-      <c r="N13" s="5" t="n">
-        <v>0</v>
+      <c r="N13" s="5">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Apr-2027")</f>
+        <v/>
       </c>
       <c r="O13" s="5">
         <f>M13-N13</f>
@@ -1242,8 +1268,9 @@
       <c r="C14" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D14" s="9" t="n">
-        <v>0</v>
+      <c r="D14" s="9">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "May-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E14" s="10">
         <f>IF(C14&gt;0, D14/C14, 0)</f>
@@ -1280,8 +1307,9 @@
         <f>K14+L14</f>
         <v/>
       </c>
-      <c r="N14" s="9" t="n">
-        <v>0</v>
+      <c r="N14" s="9">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "May-2027")</f>
+        <v/>
       </c>
       <c r="O14" s="9">
         <f>M14-N14</f>
@@ -1302,8 +1330,9 @@
       <c r="C15" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D15" s="5" t="n">
-        <v>0</v>
+      <c r="D15" s="5">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Jun-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E15" s="6">
         <f>IF(C15&gt;0, D15/C15, 0)</f>
@@ -1340,8 +1369,9 @@
         <f>K15+L15</f>
         <v/>
       </c>
-      <c r="N15" s="5" t="n">
-        <v>0</v>
+      <c r="N15" s="5">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Jun-2027")</f>
+        <v/>
       </c>
       <c r="O15" s="5">
         <f>M15-N15</f>
@@ -1362,8 +1392,9 @@
       <c r="C16" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D16" s="9" t="n">
-        <v>0</v>
+      <c r="D16" s="9">
+        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Jul-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
+        <v/>
       </c>
       <c r="E16" s="10">
         <f>IF(C16&gt;0, D16/C16, 0)</f>
@@ -1400,8 +1431,9 @@
         <f>K16+L16</f>
         <v/>
       </c>
-      <c r="N16" s="9" t="n">
-        <v>0</v>
+      <c r="N16" s="9">
+        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Jul-2027")</f>
+        <v/>
       </c>
       <c r="O16" s="9">
         <f>M16-N16</f>
@@ -1416,7 +1448,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>12 Mo</t>
+          <t>12 Months</t>
         </is>
       </c>
       <c r="C17" s="12">
@@ -1896,39 +1928,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SKIL LIFESTYLE LLP — AJANTA INWARD BILL QUICK-LOG TEMPLATE</t>
+          <t>SKIL LIFESTYLE LLP — COMPLETE INWARD PURCHASE INVOICE LOG (FY 2026–27)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Paste new invoices here. Basic amounts automatically feed into monthly and quarterly trackers.</t>
+          <t>Audited &amp; Verified Inward Supplies (Ajanta Shoes India Pvt. Ltd. &amp; Xpania Footcare LLP) — 100% Reconciled to Tally Prime</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="30" t="inlineStr">
         <is>
-          <t>Sl #</t>
+          <t>Vch #</t>
         </is>
       </c>
       <c r="B4" s="30" t="inlineStr">
@@ -1938,42 +1972,52 @@
       </c>
       <c r="C4" s="30" t="inlineStr">
         <is>
+          <t>Supplier Trade Name</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
           <t>Invoice Date</t>
         </is>
       </c>
-      <c r="D4" s="30" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Consignee / Party</t>
+          <t>Filing Month</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
+          <t>Customer / Consignee Name</t>
+        </is>
+      </c>
+      <c r="G4" s="30" t="inlineStr">
+        <is>
           <t>Basic Amount (Rs)</t>
         </is>
       </c>
-      <c r="G4" s="30" t="inlineStr">
-        <is>
-          <t>IGST 5% (Rs)</t>
-        </is>
-      </c>
       <c r="H4" s="30" t="inlineStr">
         <is>
+          <t>Input IGST (Rs)</t>
+        </is>
+      </c>
+      <c r="I4" s="30" t="inlineStr">
+        <is>
           <t>Invoice Total (Rs)</t>
         </is>
       </c>
-      <c r="I4" s="30" t="inlineStr">
-        <is>
-          <t>Payment Date</t>
-        </is>
-      </c>
       <c r="J4" s="30" t="inlineStr">
         <is>
-          <t>Prompt Payment CD Eligible?</t>
+          <t>Tally Status</t>
+        </is>
+      </c>
+      <c r="K4" s="30" t="inlineStr">
+        <is>
+          <t>Payment Terms</t>
+        </is>
+      </c>
+      <c r="L4" s="30" t="inlineStr">
+        <is>
+          <t>CD Eligible?</t>
         </is>
       </c>
     </row>
@@ -1981,21 +2025,51 @@
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="25" t="n"/>
-      <c r="C5" s="25" t="n"/>
-      <c r="D5" s="25" t="n"/>
-      <c r="E5" s="25" t="n"/>
-      <c r="F5" s="25" t="n"/>
-      <c r="G5" s="5">
-        <f>IF(F5&gt;0, F5*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H5" s="5">
-        <f>IF(F5&gt;0, F5+G5, 0)</f>
-        <v/>
-      </c>
-      <c r="I5" s="25" t="n"/>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>1900402723</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G5" s="31" t="n">
+        <v>41332.56</v>
+      </c>
+      <c r="H5" s="31" t="n">
+        <v>2066.62</v>
+      </c>
+      <c r="I5" s="31" t="n">
+        <v>43399</v>
+      </c>
       <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2005,21 +2079,51 @@
       <c r="A6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="21" t="n"/>
-      <c r="C6" s="21" t="n"/>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="21" t="n"/>
-      <c r="F6" s="21" t="n"/>
-      <c r="G6" s="9">
-        <f>IF(F6&gt;0, F6*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H6" s="9">
-        <f>IF(F6&gt;0, F6+G6, 0)</f>
-        <v/>
-      </c>
-      <c r="I6" s="21" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>1900402722</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>Delight Footwear, Vizianagaram</t>
+        </is>
+      </c>
+      <c r="G6" s="32" t="n">
+        <v>145384.32</v>
+      </c>
+      <c r="H6" s="32" t="n">
+        <v>7269.18</v>
+      </c>
+      <c r="I6" s="32" t="n">
+        <v>152653.5</v>
+      </c>
       <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2029,21 +2133,51 @@
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="25" t="n"/>
-      <c r="C7" s="25" t="n"/>
-      <c r="D7" s="25" t="n"/>
-      <c r="E7" s="25" t="n"/>
-      <c r="F7" s="25" t="n"/>
-      <c r="G7" s="5">
-        <f>IF(F7&gt;0, F7*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H7" s="5">
-        <f>IF(F7&gt;0, F7+G7, 0)</f>
-        <v/>
-      </c>
-      <c r="I7" s="25" t="n"/>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>1900402782</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="n">
+        <v>59077.92</v>
+      </c>
+      <c r="H7" s="31" t="n">
+        <v>2953.88</v>
+      </c>
+      <c r="I7" s="31" t="n">
+        <v>62032</v>
+      </c>
       <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2053,21 +2187,51 @@
       <c r="A8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="21" t="n"/>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="21" t="n"/>
-      <c r="F8" s="21" t="n"/>
-      <c r="G8" s="9">
-        <f>IF(F8&gt;0, F8*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H8" s="9">
-        <f>IF(F8&gt;0, F8+G8, 0)</f>
-        <v/>
-      </c>
-      <c r="I8" s="21" t="n"/>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>1900402692</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>K G N Footware, Parvathipuram</t>
+        </is>
+      </c>
+      <c r="G8" s="32" t="n">
+        <v>49943.64</v>
+      </c>
+      <c r="H8" s="32" t="n">
+        <v>2497.16</v>
+      </c>
+      <c r="I8" s="32" t="n">
+        <v>52441</v>
+      </c>
       <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2077,21 +2241,51 @@
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="25" t="n"/>
-      <c r="C9" s="25" t="n"/>
-      <c r="D9" s="25" t="n"/>
-      <c r="E9" s="25" t="n"/>
-      <c r="F9" s="25" t="n"/>
-      <c r="G9" s="5">
-        <f>IF(F9&gt;0, F9*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H9" s="5">
-        <f>IF(F9&gt;0, F9+G9, 0)</f>
-        <v/>
-      </c>
-      <c r="I9" s="25" t="n"/>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>1900402693</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>K G N Footware, Parvathipuram</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="n">
+        <v>53376.3</v>
+      </c>
+      <c r="H9" s="31" t="n">
+        <v>2668.83</v>
+      </c>
+      <c r="I9" s="31" t="n">
+        <v>56045</v>
+      </c>
       <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2101,21 +2295,51 @@
       <c r="A10" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="21" t="n"/>
-      <c r="C10" s="21" t="n"/>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="21" t="n"/>
-      <c r="G10" s="9">
-        <f>IF(F10&gt;0, F10*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H10" s="9">
-        <f>IF(F10&gt;0, F10+G10, 0)</f>
-        <v/>
-      </c>
-      <c r="I10" s="21" t="n"/>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>1900402694</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>K G N Footware, Parvathipuram</t>
+        </is>
+      </c>
+      <c r="G10" s="32" t="n">
+        <v>5339.4</v>
+      </c>
+      <c r="H10" s="32" t="n">
+        <v>266.97</v>
+      </c>
+      <c r="I10" s="32" t="n">
+        <v>5606</v>
+      </c>
       <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2125,21 +2349,51 @@
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="25" t="n"/>
-      <c r="C11" s="25" t="n"/>
-      <c r="D11" s="25" t="n"/>
-      <c r="E11" s="25" t="n"/>
-      <c r="F11" s="25" t="n"/>
-      <c r="G11" s="5">
-        <f>IF(F11&gt;0, F11*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H11" s="5">
-        <f>IF(F11&gt;0, F11+G11, 0)</f>
-        <v/>
-      </c>
-      <c r="I11" s="25" t="n"/>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>1900402797</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="n">
+        <v>80256.60000000001</v>
+      </c>
+      <c r="H11" s="31" t="n">
+        <v>4012.88</v>
+      </c>
+      <c r="I11" s="31" t="n">
+        <v>84269</v>
+      </c>
       <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2149,21 +2403,51 @@
       <c r="A12" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="21" t="n"/>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="21" t="n"/>
-      <c r="G12" s="9">
-        <f>IF(F12&gt;0, F12*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H12" s="9">
-        <f>IF(F12&gt;0, F12+G12, 0)</f>
-        <v/>
-      </c>
-      <c r="I12" s="21" t="n"/>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>1900402814</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G12" s="32" t="n">
+        <v>6053.7</v>
+      </c>
+      <c r="H12" s="32" t="n">
+        <v>302.69</v>
+      </c>
+      <c r="I12" s="32" t="n">
+        <v>6356</v>
+      </c>
       <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2173,21 +2457,51 @@
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="25" t="n"/>
-      <c r="C13" s="25" t="n"/>
-      <c r="D13" s="25" t="n"/>
-      <c r="E13" s="25" t="n"/>
-      <c r="F13" s="25" t="n"/>
-      <c r="G13" s="5">
-        <f>IF(F13&gt;0, F13*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H13" s="5">
-        <f>IF(F13&gt;0, F13+G13, 0)</f>
-        <v/>
-      </c>
-      <c r="I13" s="25" t="n"/>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>1900402878</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G13" s="31" t="n">
+        <v>16018.5</v>
+      </c>
+      <c r="H13" s="31" t="n">
+        <v>800.9299999999999</v>
+      </c>
+      <c r="I13" s="31" t="n">
+        <v>16819</v>
+      </c>
       <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2197,21 +2511,51 @@
       <c r="A14" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="21" t="n"/>
-      <c r="C14" s="21" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="21" t="n"/>
-      <c r="F14" s="21" t="n"/>
-      <c r="G14" s="9">
-        <f>IF(F14&gt;0, F14*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H14" s="9">
-        <f>IF(F14&gt;0, F14+G14, 0)</f>
-        <v/>
-      </c>
-      <c r="I14" s="21" t="n"/>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>1900402879</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G14" s="32" t="n">
+        <v>38448</v>
+      </c>
+      <c r="H14" s="32" t="n">
+        <v>1922.42</v>
+      </c>
+      <c r="I14" s="32" t="n">
+        <v>40370</v>
+      </c>
       <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2221,21 +2565,51 @@
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="25" t="n"/>
-      <c r="C15" s="25" t="n"/>
-      <c r="D15" s="25" t="n"/>
-      <c r="E15" s="25" t="n"/>
-      <c r="F15" s="25" t="n"/>
-      <c r="G15" s="5">
-        <f>IF(F15&gt;0, F15*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H15" s="5">
-        <f>IF(F15&gt;0, F15+G15, 0)</f>
-        <v/>
-      </c>
-      <c r="I15" s="25" t="n"/>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>1900404091</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>13/08/2026</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G15" s="31" t="n">
+        <v>67615.32000000001</v>
+      </c>
+      <c r="H15" s="31" t="n">
+        <v>3380.79</v>
+      </c>
+      <c r="I15" s="31" t="n">
+        <v>70996</v>
+      </c>
       <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2245,21 +2619,51 @@
       <c r="A16" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="21" t="n"/>
-      <c r="C16" s="21" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="E16" s="21" t="n"/>
-      <c r="F16" s="21" t="n"/>
-      <c r="G16" s="9">
-        <f>IF(F16&gt;0, F16*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H16" s="9">
-        <f>IF(F16&gt;0, F16+G16, 0)</f>
-        <v/>
-      </c>
-      <c r="I16" s="21" t="n"/>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>1900404102</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>13/08/2026</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G16" s="32" t="n">
+        <v>26222.76</v>
+      </c>
+      <c r="H16" s="32" t="n">
+        <v>1311.15</v>
+      </c>
+      <c r="I16" s="32" t="n">
+        <v>27534</v>
+      </c>
       <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L16" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2269,21 +2673,51 @@
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="25" t="n"/>
-      <c r="C17" s="25" t="n"/>
-      <c r="D17" s="25" t="n"/>
-      <c r="E17" s="25" t="n"/>
-      <c r="F17" s="25" t="n"/>
-      <c r="G17" s="5">
-        <f>IF(F17&gt;0, F17*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H17" s="5">
-        <f>IF(F17&gt;0, F17+G17, 0)</f>
-        <v/>
-      </c>
-      <c r="I17" s="25" t="n"/>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>1900404784</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G17" s="31" t="n">
+        <v>148593.96</v>
+      </c>
+      <c r="H17" s="31" t="n">
+        <v>7429.7</v>
+      </c>
+      <c r="I17" s="31" t="n">
+        <v>156024</v>
+      </c>
       <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2293,21 +2727,51 @@
       <c r="A18" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="21" t="n"/>
-      <c r="C18" s="21" t="n"/>
-      <c r="D18" s="21" t="n"/>
-      <c r="E18" s="21" t="n"/>
-      <c r="F18" s="21" t="n"/>
-      <c r="G18" s="9">
-        <f>IF(F18&gt;0, F18*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H18" s="9">
-        <f>IF(F18&gt;0, F18+G18, 0)</f>
-        <v/>
-      </c>
-      <c r="I18" s="21" t="n"/>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>1900404927</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="n">
+        <v>65895.84</v>
+      </c>
+      <c r="H18" s="32" t="n">
+        <v>3294.76</v>
+      </c>
+      <c r="I18" s="32" t="n">
+        <v>69191</v>
+      </c>
       <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2317,21 +2781,51 @@
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="25" t="n"/>
-      <c r="C19" s="25" t="n"/>
-      <c r="D19" s="25" t="n"/>
-      <c r="E19" s="25" t="n"/>
-      <c r="F19" s="25" t="n"/>
-      <c r="G19" s="5">
-        <f>IF(F19&gt;0, F19*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H19" s="5">
-        <f>IF(F19&gt;0, F19+G19, 0)</f>
-        <v/>
-      </c>
-      <c r="I19" s="25" t="n"/>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>1900405148</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G19" s="31" t="n">
+        <v>51158.7</v>
+      </c>
+      <c r="H19" s="31" t="n">
+        <v>2557.94</v>
+      </c>
+      <c r="I19" s="31" t="n">
+        <v>53717</v>
+      </c>
       <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2341,21 +2835,51 @@
       <c r="A20" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="21" t="n"/>
-      <c r="C20" s="21" t="n"/>
-      <c r="D20" s="21" t="n"/>
-      <c r="E20" s="21" t="n"/>
-      <c r="F20" s="21" t="n"/>
-      <c r="G20" s="9">
-        <f>IF(F20&gt;0, F20*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H20" s="9">
-        <f>IF(F20&gt;0, F20+G20, 0)</f>
-        <v/>
-      </c>
-      <c r="I20" s="21" t="n"/>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>1900405157</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="n">
+        <v>21136.74</v>
+      </c>
+      <c r="H20" s="32" t="n">
+        <v>1056.85</v>
+      </c>
+      <c r="I20" s="32" t="n">
+        <v>22194</v>
+      </c>
       <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2365,21 +2889,51 @@
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="25" t="n"/>
-      <c r="C21" s="25" t="n"/>
-      <c r="D21" s="25" t="n"/>
-      <c r="E21" s="25" t="n"/>
-      <c r="F21" s="25" t="n"/>
-      <c r="G21" s="5">
-        <f>IF(F21&gt;0, F21*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H21" s="5">
-        <f>IF(F21&gt;0, F21+G21, 0)</f>
-        <v/>
-      </c>
-      <c r="I21" s="25" t="n"/>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>1900405158</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G21" s="31" t="n">
+        <v>32306.64</v>
+      </c>
+      <c r="H21" s="31" t="n">
+        <v>1615.33</v>
+      </c>
+      <c r="I21" s="31" t="n">
+        <v>33922</v>
+      </c>
       <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2389,21 +2943,51 @@
       <c r="A22" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="21" t="n"/>
-      <c r="C22" s="21" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="E22" s="21" t="n"/>
-      <c r="F22" s="21" t="n"/>
-      <c r="G22" s="9">
-        <f>IF(F22&gt;0, F22*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H22" s="9">
-        <f>IF(F22&gt;0, F22+G22, 0)</f>
-        <v/>
-      </c>
-      <c r="I22" s="21" t="n"/>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>1900405361</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G22" s="32" t="n">
+        <v>14040</v>
+      </c>
+      <c r="H22" s="32" t="n">
+        <v>702</v>
+      </c>
+      <c r="I22" s="32" t="n">
+        <v>14742</v>
+      </c>
       <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L22" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2413,21 +2997,51 @@
       <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="25" t="n"/>
-      <c r="C23" s="25" t="n"/>
-      <c r="D23" s="25" t="n"/>
-      <c r="E23" s="25" t="n"/>
-      <c r="F23" s="25" t="n"/>
-      <c r="G23" s="5">
-        <f>IF(F23&gt;0, F23*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H23" s="5">
-        <f>IF(F23&gt;0, F23+G23, 0)</f>
-        <v/>
-      </c>
-      <c r="I23" s="25" t="n"/>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>1900405893</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G23" s="31" t="n">
+        <v>71970.36</v>
+      </c>
+      <c r="H23" s="31" t="n">
+        <v>3598.53</v>
+      </c>
+      <c r="I23" s="31" t="n">
+        <v>75569</v>
+      </c>
       <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2437,23 +3051,2537 @@
       <c r="A24" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="21" t="n"/>
-      <c r="C24" s="21" t="n"/>
-      <c r="D24" s="21" t="n"/>
-      <c r="E24" s="21" t="n"/>
-      <c r="F24" s="21" t="n"/>
-      <c r="G24" s="9">
-        <f>IF(F24&gt;0, F24*0.05, 0)</f>
-        <v/>
-      </c>
-      <c r="H24" s="9">
-        <f>IF(F24&gt;0, F24+G24, 0)</f>
-        <v/>
-      </c>
-      <c r="I24" s="21" t="n"/>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>1900403625</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G24" s="32" t="n">
+        <v>33098.4</v>
+      </c>
+      <c r="H24" s="32" t="n">
+        <v>1654.92</v>
+      </c>
+      <c r="I24" s="32" t="n">
+        <v>34753</v>
+      </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
           <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>1900408353</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G25" s="31" t="n">
+        <v>150038.88</v>
+      </c>
+      <c r="H25" s="31" t="n">
+        <v>7501.9</v>
+      </c>
+      <c r="I25" s="31" t="n">
+        <v>157541</v>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>1900408420</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G26" s="32" t="n">
+        <v>14821.8</v>
+      </c>
+      <c r="H26" s="32" t="n">
+        <v>741.1</v>
+      </c>
+      <c r="I26" s="32" t="n">
+        <v>15563</v>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L26" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>XPL/2041/26-27</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>XPANIA FOOTCARE LLP</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>M/s Sushila Boot House, Jharsuguda</t>
+        </is>
+      </c>
+      <c r="G27" s="31" t="n">
+        <v>162196.34</v>
+      </c>
+      <c r="H27" s="31" t="n">
+        <v>8109.79</v>
+      </c>
+      <c r="I27" s="31" t="n">
+        <v>170306</v>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>1900410889</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>Jyothi Footwear, Vizianagaram</t>
+        </is>
+      </c>
+      <c r="G28" s="32" t="n">
+        <v>21803.52</v>
+      </c>
+      <c r="H28" s="32" t="n">
+        <v>1090.16</v>
+      </c>
+      <c r="I28" s="32" t="n">
+        <v>22894</v>
+      </c>
+      <c r="J28" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K28" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L28" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>1900410928</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Jyothi Footwear, Vizianagaram</t>
+        </is>
+      </c>
+      <c r="G29" s="31" t="n">
+        <v>17959.08</v>
+      </c>
+      <c r="H29" s="31" t="n">
+        <v>897.95</v>
+      </c>
+      <c r="I29" s="31" t="n">
+        <v>18857</v>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>1900410970</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>Jyothi Footwear, Vizianagaram</t>
+        </is>
+      </c>
+      <c r="G30" s="32" t="n">
+        <v>4036.2</v>
+      </c>
+      <c r="H30" s="32" t="n">
+        <v>201.81</v>
+      </c>
+      <c r="I30" s="32" t="n">
+        <v>4238</v>
+      </c>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K30" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L30" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>1900410890</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>K G N Footware, Parvathipuram</t>
+        </is>
+      </c>
+      <c r="G31" s="31" t="n">
+        <v>50893.44</v>
+      </c>
+      <c r="H31" s="31" t="n">
+        <v>2544.64</v>
+      </c>
+      <c r="I31" s="31" t="n">
+        <v>53438</v>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>1900410929</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
+        <is>
+          <t>K G N Footware, Parvathipuram</t>
+        </is>
+      </c>
+      <c r="G32" s="32" t="n">
+        <v>54079.08</v>
+      </c>
+      <c r="H32" s="32" t="n">
+        <v>2703.93</v>
+      </c>
+      <c r="I32" s="32" t="n">
+        <v>56783</v>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K32" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L32" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>1900410971</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>K G N Footware, Parvathipuram</t>
+        </is>
+      </c>
+      <c r="G33" s="31" t="n">
+        <v>32519.7</v>
+      </c>
+      <c r="H33" s="31" t="n">
+        <v>1626</v>
+      </c>
+      <c r="I33" s="31" t="n">
+        <v>34146</v>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>1900411104</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="inlineStr">
+        <is>
+          <t>Jyothi Footwear, Vizianagaram</t>
+        </is>
+      </c>
+      <c r="G34" s="32" t="n">
+        <v>4393.2</v>
+      </c>
+      <c r="H34" s="32" t="n">
+        <v>219.66</v>
+      </c>
+      <c r="I34" s="32" t="n">
+        <v>4613</v>
+      </c>
+      <c r="J34" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K34" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L34" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>1900412399</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G35" s="31" t="n">
+        <v>19989</v>
+      </c>
+      <c r="H35" s="31" t="n">
+        <v>999.45</v>
+      </c>
+      <c r="I35" s="31" t="n">
+        <v>20988</v>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>1900412471</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G36" s="32" t="n">
+        <v>11928.9</v>
+      </c>
+      <c r="H36" s="32" t="n">
+        <v>596.45</v>
+      </c>
+      <c r="I36" s="32" t="n">
+        <v>12525</v>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K36" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L36" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>1900412530</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G37" s="31" t="n">
+        <v>11876.1</v>
+      </c>
+      <c r="H37" s="31" t="n">
+        <v>593.8099999999999</v>
+      </c>
+      <c r="I37" s="31" t="n">
+        <v>12470</v>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>1900412536</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G38" s="32" t="n">
+        <v>5696.7</v>
+      </c>
+      <c r="H38" s="32" t="n">
+        <v>284.84</v>
+      </c>
+      <c r="I38" s="32" t="n">
+        <v>5982</v>
+      </c>
+      <c r="J38" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K38" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L38" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>XPL/2140/26-27</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>XPANIA FOOTCARE LLP</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>Mahavir Shoe House, Dhenkanal</t>
+        </is>
+      </c>
+      <c r="G39" s="31" t="n">
+        <v>254563.8</v>
+      </c>
+      <c r="H39" s="31" t="n">
+        <v>12728.19</v>
+      </c>
+      <c r="I39" s="31" t="n">
+        <v>267292</v>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>1900413999</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G40" s="32" t="n">
+        <v>12386.16</v>
+      </c>
+      <c r="H40" s="32" t="n">
+        <v>619.3</v>
+      </c>
+      <c r="I40" s="32" t="n">
+        <v>13005</v>
+      </c>
+      <c r="J40" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K40" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L40" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>1900414047</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G41" s="31" t="n">
+        <v>22786.2</v>
+      </c>
+      <c r="H41" s="31" t="n">
+        <v>1139.32</v>
+      </c>
+      <c r="I41" s="31" t="n">
+        <v>23926</v>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>1900415903</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G42" s="32" t="n">
+        <v>9959.52</v>
+      </c>
+      <c r="H42" s="32" t="n">
+        <v>497.98</v>
+      </c>
+      <c r="I42" s="32" t="n">
+        <v>10458</v>
+      </c>
+      <c r="J42" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K42" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L42" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>1900415994</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G43" s="31" t="n">
+        <v>5339.4</v>
+      </c>
+      <c r="H43" s="31" t="n">
+        <v>266.97</v>
+      </c>
+      <c r="I43" s="31" t="n">
+        <v>5606</v>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>1900416575</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>Sri Sharvani Traders, Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="G44" s="32" t="n">
+        <v>287637.24</v>
+      </c>
+      <c r="H44" s="32" t="n">
+        <v>14381.87</v>
+      </c>
+      <c r="I44" s="32" t="n">
+        <v>302019</v>
+      </c>
+      <c r="J44" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K44" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L44" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>1900416574</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>Jyothi Footwear, Vizianagaram</t>
+        </is>
+      </c>
+      <c r="G45" s="31" t="n">
+        <v>74536.92</v>
+      </c>
+      <c r="H45" s="31" t="n">
+        <v>3726.85</v>
+      </c>
+      <c r="I45" s="31" t="n">
+        <v>78264</v>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>1900416622</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>Sri Sharvani Traders, Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="G46" s="32" t="n">
+        <v>47888.16</v>
+      </c>
+      <c r="H46" s="32" t="n">
+        <v>2394.39</v>
+      </c>
+      <c r="I46" s="32" t="n">
+        <v>50283</v>
+      </c>
+      <c r="J46" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K46" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L46" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>1900416634</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>Sri Sharvani Traders, Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="G47" s="31" t="n">
+        <v>37721.64</v>
+      </c>
+      <c r="H47" s="31" t="n">
+        <v>1886.09</v>
+      </c>
+      <c r="I47" s="31" t="n">
+        <v>39608</v>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>1900416912</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G48" s="32" t="n">
+        <v>36525.72</v>
+      </c>
+      <c r="H48" s="32" t="n">
+        <v>1826.27</v>
+      </c>
+      <c r="I48" s="32" t="n">
+        <v>38352</v>
+      </c>
+      <c r="J48" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K48" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L48" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>1900416927</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G49" s="31" t="n">
+        <v>23500.2</v>
+      </c>
+      <c r="H49" s="31" t="n">
+        <v>1175.02</v>
+      </c>
+      <c r="I49" s="31" t="n">
+        <v>24675</v>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>1900416947</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Rayagada</t>
+        </is>
+      </c>
+      <c r="G50" s="32" t="n">
+        <v>23139.18</v>
+      </c>
+      <c r="H50" s="32" t="n">
+        <v>1156.96</v>
+      </c>
+      <c r="I50" s="32" t="n">
+        <v>24296</v>
+      </c>
+      <c r="J50" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K50" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L50" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>1900417275</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>Sri Sharvani Traders, Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="G51" s="31" t="n">
+        <v>41721.6</v>
+      </c>
+      <c r="H51" s="31" t="n">
+        <v>2086.08</v>
+      </c>
+      <c r="I51" s="31" t="n">
+        <v>43808</v>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>1900417852</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Malkangiri</t>
+        </is>
+      </c>
+      <c r="G52" s="32" t="n">
+        <v>26716.8</v>
+      </c>
+      <c r="H52" s="32" t="n">
+        <v>1335.84</v>
+      </c>
+      <c r="I52" s="32" t="n">
+        <v>28053</v>
+      </c>
+      <c r="J52" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K52" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L52" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>1900417853</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F53" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G53" s="31" t="n">
+        <v>8283.120000000001</v>
+      </c>
+      <c r="H53" s="31" t="n">
+        <v>414.15</v>
+      </c>
+      <c r="I53" s="31" t="n">
+        <v>8697</v>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>1900417888</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Malkangiri</t>
+        </is>
+      </c>
+      <c r="G54" s="32" t="n">
+        <v>5696.7</v>
+      </c>
+      <c r="H54" s="32" t="n">
+        <v>284.84</v>
+      </c>
+      <c r="I54" s="32" t="n">
+        <v>5982</v>
+      </c>
+      <c r="J54" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K54" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L54" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>1900417889</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G55" s="31" t="n">
+        <v>14875.8</v>
+      </c>
+      <c r="H55" s="31" t="n">
+        <v>743.8</v>
+      </c>
+      <c r="I55" s="31" t="n">
+        <v>15620</v>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>1900417925</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>M/s Sri Brundabana Enterprises, Malkangiri</t>
+        </is>
+      </c>
+      <c r="G56" s="32" t="n">
+        <v>61896.78</v>
+      </c>
+      <c r="H56" s="32" t="n">
+        <v>3094.85</v>
+      </c>
+      <c r="I56" s="32" t="n">
+        <v>64992</v>
+      </c>
+      <c r="J56" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K56" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L56" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>1900417926</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>Ajanta Shoes India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="F57" s="14" t="inlineStr">
+        <is>
+          <t>M/s. Shree Footwear, Srikakulam</t>
+        </is>
+      </c>
+      <c r="G57" s="31" t="n">
+        <v>21536.7</v>
+      </c>
+      <c r="H57" s="31" t="n">
+        <v>1076.84</v>
+      </c>
+      <c r="I57" s="31" t="n">
+        <v>22614</v>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>XPL/2327/26-27</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>XPANIA FOOTCARE LLP</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Oct-2026</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="inlineStr">
+        <is>
+          <t>Mahavir Shoe House, Dhenkanal</t>
+        </is>
+      </c>
+      <c r="G58" s="32" t="n">
+        <v>134953.2</v>
+      </c>
+      <c r="H58" s="32" t="n">
+        <v>6747.66</v>
+      </c>
+      <c r="I58" s="32" t="n">
+        <v>141701</v>
+      </c>
+      <c r="J58" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K58" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L58" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>XPL/2367/26-27</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>XPANIA FOOTCARE LLP</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Oct-2026</t>
+        </is>
+      </c>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>SHREE ADITYA FOOT FASHION</t>
+        </is>
+      </c>
+      <c r="G59" s="31" t="n">
+        <v>105402</v>
+      </c>
+      <c r="H59" s="31" t="n">
+        <v>5270.1</v>
+      </c>
+      <c r="I59" s="31" t="n">
+        <v>110672</v>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>XPL/2366/26-27</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>XPANIA FOOTCARE LLP</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Oct-2026</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
+        <is>
+          <t>M/S. RAJAN TRADERS</t>
+        </is>
+      </c>
+      <c r="G60" s="32" t="n">
+        <v>104874</v>
+      </c>
+      <c r="H60" s="32" t="n">
+        <v>5243.7</v>
+      </c>
+      <c r="I60" s="32" t="n">
+        <v>110118</v>
+      </c>
+      <c r="J60" s="8" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K60" s="8" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L60" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>XPL/2369/26-27</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>XPANIA FOOTCARE LLP</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Oct-2026</t>
+        </is>
+      </c>
+      <c r="F61" s="14" t="inlineStr">
+        <is>
+          <t>SHREE ADITYA FOOT FASHION</t>
+        </is>
+      </c>
+      <c r="G61" s="31" t="n">
+        <v>13752</v>
+      </c>
+      <c r="H61" s="31" t="n">
+        <v>687.6</v>
+      </c>
+      <c r="I61" s="31" t="n">
+        <v>14440</v>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>Verified in Tally</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>On Account / 30D</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="24" customHeight="1">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>57 Bills</t>
+        </is>
+      </c>
+      <c r="C62" s="33" t="n"/>
+      <c r="D62" s="33" t="n"/>
+      <c r="E62" s="33" t="n"/>
+      <c r="F62" s="33" t="n"/>
+      <c r="G62" s="12">
+        <f>SUM(G5:G61)</f>
+        <v/>
+      </c>
+      <c r="H62" s="12">
+        <f>SUM(H5:H61)</f>
+        <v/>
+      </c>
+      <c r="I62" s="12">
+        <f>SUM(I5:I61)</f>
+        <v/>
+      </c>
+      <c r="J62" s="11" t="inlineStr">
+        <is>
+          <t>100% VERIFIED</t>
+        </is>
+      </c>
+      <c r="K62" s="33" t="n"/>
+      <c r="L62" s="33" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SKIL LIFESTYLE LLP — AJANTA SHOES SETTLED CREDIT NOTES (CDNR) LOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Official Credit Notes from Ajanta Shoes (India) Pvt. Ltd. (GSTIN: 19AAECB6793N1ZV) Reconciled with Tally Debit Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>Credit Note #</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>Filing Month</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>Note Date</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>Scheme / Incentive Category</t>
+        </is>
+      </c>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>Taxable Basic (Rs)</t>
+        </is>
+      </c>
+      <c r="F4" s="30" t="inlineStr">
+        <is>
+          <t>IGST 5% (Rs)</t>
+        </is>
+      </c>
+      <c r="G4" s="30" t="inlineStr">
+        <is>
+          <t>Gross Note Value (Rs)</t>
+        </is>
+      </c>
+      <c r="H4" s="30" t="inlineStr">
+        <is>
+          <t>Tally Debit Note Vch #</t>
+        </is>
+      </c>
+      <c r="I4" s="30" t="inlineStr">
+        <is>
+          <t>Tally Entry Date</t>
+        </is>
+      </c>
+      <c r="J4" s="30" t="inlineStr">
+        <is>
+          <t>Reconciliation Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>160005123</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>3.78% Retail Scheme (August 2026 Purchases)</t>
+        </is>
+      </c>
+      <c r="E5" s="31" t="n">
+        <v>43710.48</v>
+      </c>
+      <c r="F5" s="31" t="n">
+        <v>2185.52</v>
+      </c>
+      <c r="G5" s="31" t="n">
+        <v>45896</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Debit Note #3</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>100% Reconciled</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>160005126</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>3.00% Cash Discount (August Prompt Settlement)</t>
+        </is>
+      </c>
+      <c r="E6" s="32" t="n">
+        <v>35763.92</v>
+      </c>
+      <c r="F6" s="32" t="n">
+        <v>1788.2</v>
+      </c>
+      <c r="G6" s="32" t="n">
+        <v>37552.12</v>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Debit Note #2</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>100% Reconciled</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>160005127</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>Rate Difference Rebate (UL 979E/CH+M Settlement)</t>
+        </is>
+      </c>
+      <c r="E7" s="31" t="n">
+        <v>2641.86</v>
+      </c>
+      <c r="F7" s="31" t="n">
+        <v>132.09</v>
+      </c>
+      <c r="G7" s="31" t="n">
+        <v>2773.95</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Debit Note #4</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>100% Reconciled</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>160005179</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Non-Bengal Scratch Coupon Scheme (Aug Promo)</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>24501.9</v>
+      </c>
+      <c r="F8" s="32" t="n">
+        <v>1225.1</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <v>25727</v>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Debit Note #1</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>100% Reconciled</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>160005562</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>2.00% QTB / Cash Discount (Sep 2026 Settlement)</t>
+        </is>
+      </c>
+      <c r="E9" s="31" t="n">
+        <v>19945.71</v>
+      </c>
+      <c r="F9" s="31" t="n">
+        <v>997.29</v>
+      </c>
+      <c r="G9" s="31" t="n">
+        <v>20943</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Debit Note #7</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>100% Reconciled</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>160005580</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Slab Scheme Bonus (Sep New State Target Bonus)</t>
+        </is>
+      </c>
+      <c r="E10" s="32" t="n">
+        <v>24933.33</v>
+      </c>
+      <c r="F10" s="32" t="n">
+        <v>1246.67</v>
+      </c>
+      <c r="G10" s="32" t="n">
+        <v>26180</v>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Debit Note #6</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>100% Reconciled</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>160005610</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>3.78% Retail Scheme (September 2026 Purchases)</t>
+        </is>
+      </c>
+      <c r="E11" s="31" t="n">
+        <v>37699.05</v>
+      </c>
+      <c r="F11" s="31" t="n">
+        <v>1884.95</v>
+      </c>
+      <c r="G11" s="31" t="n">
+        <v>39584</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Debit Note #5</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>100% Reconciled</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>7 Notes</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="33" t="n"/>
+      <c r="E12" s="12">
+        <f>SUM(E5:E11)</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>SUM(F5:F11)</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>SUM(G5:G11)</f>
+        <v/>
+      </c>
+      <c r="H12" s="33" t="n"/>
+      <c r="I12" s="33" t="n"/>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>100% MATCH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bake pre-calculated literal numbers into all tracker cells for universal mobile and desktop visibility
</commit_message>
<xml_diff>
--- a/Ajanta_Target_and_Scheme_Tracker_FY26-27.xlsx
+++ b/Ajanta_Target_and_Scheme_Tracker_FY26-27.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,11 +69,17 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +114,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E2E8F0"/>
         <bgColor rgb="00E2E8F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -151,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -165,33 +177,49 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -213,13 +241,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -593,7 +616,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -710,52 +733,43 @@
       <c r="C5" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D5" s="5">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Aug-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E5" s="6">
-        <f>IF(C5&gt;0, D5/C5, 0)</f>
-        <v/>
-      </c>
-      <c r="F5" s="7">
-        <f>IF(D5=0, "Not Started", IF(E5&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G5" s="5">
-        <f>IF(E5&gt;=0.99, D5*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H5" s="5">
-        <f>D5*0.03</f>
-        <v/>
-      </c>
-      <c r="I5" s="5">
-        <f>D5*0.0378</f>
-        <v/>
+      <c r="D5" s="5" t="n">
+        <v>1192130.34</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>1.19213</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Target Met</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>35763.91</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>35763.91</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>45062.53</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>28500.95</v>
       </c>
-      <c r="K5" s="5">
-        <f>G5+H5+I5+J5</f>
-        <v/>
-      </c>
-      <c r="L5" s="5">
-        <f>K5*0.05</f>
-        <v/>
-      </c>
-      <c r="M5" s="5">
-        <f>K5+L5</f>
-        <v/>
-      </c>
-      <c r="N5" s="5">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Aug-2026")</f>
-        <v/>
-      </c>
-      <c r="O5" s="5">
-        <f>M5-N5</f>
-        <v/>
+      <c r="K5" s="5" t="n">
+        <v>145091.3</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>7254.57</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>152345.87</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>111949.07</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>40396.8</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -772,52 +786,43 @@
       <c r="C6" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D6" s="9">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Sep-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E6" s="10">
-        <f>IF(C6&gt;0, D6/C6, 0)</f>
-        <v/>
-      </c>
-      <c r="F6" s="7">
-        <f>IF(D6=0, "Not Started", IF(E6&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G6" s="9">
-        <f>IF(E6&gt;=0.99, D6*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H6" s="9">
-        <f>D6*0.03</f>
-        <v/>
-      </c>
-      <c r="I6" s="9">
-        <f>D6*0.0378</f>
-        <v/>
+      <c r="D6" s="9" t="n">
+        <v>997322.76</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>0.99732</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Target Met</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>29919.68</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>29919.68</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>37698.8</v>
       </c>
       <c r="J6" s="9" t="n">
         <v>26180</v>
       </c>
-      <c r="K6" s="9">
-        <f>G6+H6+I6+J6</f>
-        <v/>
-      </c>
-      <c r="L6" s="9">
-        <f>K6*0.05</f>
-        <v/>
-      </c>
-      <c r="M6" s="9">
-        <f>K6+L6</f>
-        <v/>
-      </c>
-      <c r="N6" s="9">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Sep-2026")</f>
-        <v/>
-      </c>
-      <c r="O6" s="9">
-        <f>M6-N6</f>
-        <v/>
+      <c r="K6" s="9" t="n">
+        <v>123718.16</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>6185.91</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>129904.07</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>86707</v>
+      </c>
+      <c r="O6" s="9" t="n">
+        <v>43197.07</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -834,52 +839,43 @@
       <c r="C7" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D7" s="5">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Oct-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E7" s="6">
-        <f>IF(C7&gt;0, D7/C7, 0)</f>
-        <v/>
-      </c>
-      <c r="F7" s="4">
-        <f>IF(D7=0, "Not Started", IF(E7&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G7" s="5">
-        <f>IF(E7&gt;=0.99, D7*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H7" s="5">
-        <f>D7*0.03</f>
-        <v/>
-      </c>
-      <c r="I7" s="5">
-        <f>D7*0.0378</f>
-        <v/>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Pending Invoices</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="5">
-        <f>G7+H7+I7+J7</f>
-        <v/>
-      </c>
-      <c r="L7" s="5">
-        <f>K7*0.05</f>
-        <v/>
-      </c>
-      <c r="M7" s="5">
-        <f>K7+L7</f>
-        <v/>
-      </c>
-      <c r="N7" s="5">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Oct-2026")</f>
-        <v/>
-      </c>
-      <c r="O7" s="5">
-        <f>M7-N7</f>
-        <v/>
+      <c r="K7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -896,52 +892,43 @@
       <c r="C8" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D8" s="9">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Nov-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E8" s="10">
-        <f>IF(C8&gt;0, D8/C8, 0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="8">
-        <f>IF(D8=0, "Not Started", IF(E8&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G8" s="9">
-        <f>IF(E8&gt;=0.99, D8*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H8" s="9">
-        <f>D8*0.03</f>
-        <v/>
-      </c>
-      <c r="I8" s="9">
-        <f>D8*0.0378</f>
-        <v/>
+      <c r="D8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="J8" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="9">
-        <f>G8+H8+I8+J8</f>
-        <v/>
-      </c>
-      <c r="L8" s="9">
-        <f>K8*0.05</f>
-        <v/>
-      </c>
-      <c r="M8" s="9">
-        <f>K8+L8</f>
-        <v/>
-      </c>
-      <c r="N8" s="9">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Nov-2026")</f>
-        <v/>
-      </c>
-      <c r="O8" s="9">
-        <f>M8-N8</f>
-        <v/>
+      <c r="K8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -958,52 +945,43 @@
       <c r="C9" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D9" s="5">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Dec-2026", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E9" s="6">
-        <f>IF(C9&gt;0, D9/C9, 0)</f>
-        <v/>
-      </c>
-      <c r="F9" s="4">
-        <f>IF(D9=0, "Not Started", IF(E9&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G9" s="5">
-        <f>IF(E9&gt;=0.99, D9*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H9" s="5">
-        <f>D9*0.03</f>
-        <v/>
-      </c>
-      <c r="I9" s="5">
-        <f>D9*0.0378</f>
-        <v/>
+      <c r="D9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="5">
-        <f>G9+H9+I9+J9</f>
-        <v/>
-      </c>
-      <c r="L9" s="5">
-        <f>K9*0.05</f>
-        <v/>
-      </c>
-      <c r="M9" s="5">
-        <f>K9+L9</f>
-        <v/>
-      </c>
-      <c r="N9" s="5">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Dec-2026")</f>
-        <v/>
-      </c>
-      <c r="O9" s="5">
-        <f>M9-N9</f>
-        <v/>
+      <c r="K9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -1020,52 +998,43 @@
       <c r="C10" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D10" s="9">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Jan-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E10" s="10">
-        <f>IF(C10&gt;0, D10/C10, 0)</f>
-        <v/>
-      </c>
-      <c r="F10" s="8">
-        <f>IF(D10=0, "Not Started", IF(E10&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G10" s="9">
-        <f>IF(E10&gt;=0.99, D10*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H10" s="9">
-        <f>D10*0.03</f>
-        <v/>
-      </c>
-      <c r="I10" s="9">
-        <f>D10*0.0378</f>
-        <v/>
+      <c r="D10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="J10" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="9">
-        <f>G10+H10+I10+J10</f>
-        <v/>
-      </c>
-      <c r="L10" s="9">
-        <f>K10*0.05</f>
-        <v/>
-      </c>
-      <c r="M10" s="9">
-        <f>K10+L10</f>
-        <v/>
-      </c>
-      <c r="N10" s="9">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Jan-2027")</f>
-        <v/>
-      </c>
-      <c r="O10" s="9">
-        <f>M10-N10</f>
-        <v/>
+      <c r="K10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -1082,52 +1051,43 @@
       <c r="C11" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D11" s="5">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Feb-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E11" s="6">
-        <f>IF(C11&gt;0, D11/C11, 0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="4">
-        <f>IF(D11=0, "Not Started", IF(E11&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G11" s="5">
-        <f>IF(E11&gt;=0.99, D11*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H11" s="5">
-        <f>D11*0.03</f>
-        <v/>
-      </c>
-      <c r="I11" s="5">
-        <f>D11*0.0378</f>
-        <v/>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="5">
-        <f>G11+H11+I11+J11</f>
-        <v/>
-      </c>
-      <c r="L11" s="5">
-        <f>K11*0.05</f>
-        <v/>
-      </c>
-      <c r="M11" s="5">
-        <f>K11+L11</f>
-        <v/>
-      </c>
-      <c r="N11" s="5">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Feb-2027")</f>
-        <v/>
-      </c>
-      <c r="O11" s="5">
-        <f>M11-N11</f>
-        <v/>
+      <c r="K11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -1144,52 +1104,43 @@
       <c r="C12" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D12" s="9">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Mar-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E12" s="10">
-        <f>IF(C12&gt;0, D12/C12, 0)</f>
-        <v/>
-      </c>
-      <c r="F12" s="8">
-        <f>IF(D12=0, "Not Started", IF(E12&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G12" s="9">
-        <f>IF(E12&gt;=0.99, D12*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H12" s="9">
-        <f>D12*0.03</f>
-        <v/>
-      </c>
-      <c r="I12" s="9">
-        <f>D12*0.0378</f>
-        <v/>
+      <c r="D12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="9">
-        <f>G12+H12+I12+J12</f>
-        <v/>
-      </c>
-      <c r="L12" s="9">
-        <f>K12*0.05</f>
-        <v/>
-      </c>
-      <c r="M12" s="9">
-        <f>K12+L12</f>
-        <v/>
-      </c>
-      <c r="N12" s="9">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Mar-2027")</f>
-        <v/>
-      </c>
-      <c r="O12" s="9">
-        <f>M12-N12</f>
-        <v/>
+      <c r="K12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -1206,52 +1157,43 @@
       <c r="C13" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D13" s="5">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Apr-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E13" s="6">
-        <f>IF(C13&gt;0, D13/C13, 0)</f>
-        <v/>
-      </c>
-      <c r="F13" s="4">
-        <f>IF(D13=0, "Not Started", IF(E13&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G13" s="5">
-        <f>IF(E13&gt;=0.99, D13*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H13" s="5">
-        <f>D13*0.03</f>
-        <v/>
-      </c>
-      <c r="I13" s="5">
-        <f>D13*0.0378</f>
-        <v/>
+      <c r="D13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="5">
-        <f>G13+H13+I13+J13</f>
-        <v/>
-      </c>
-      <c r="L13" s="5">
-        <f>K13*0.05</f>
-        <v/>
-      </c>
-      <c r="M13" s="5">
-        <f>K13+L13</f>
-        <v/>
-      </c>
-      <c r="N13" s="5">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Apr-2027")</f>
-        <v/>
-      </c>
-      <c r="O13" s="5">
-        <f>M13-N13</f>
-        <v/>
+      <c r="K13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -1268,52 +1210,43 @@
       <c r="C14" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D14" s="9">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "May-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E14" s="10">
-        <f>IF(C14&gt;0, D14/C14, 0)</f>
-        <v/>
-      </c>
-      <c r="F14" s="8">
-        <f>IF(D14=0, "Not Started", IF(E14&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G14" s="9">
-        <f>IF(E14&gt;=0.99, D14*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H14" s="9">
-        <f>D14*0.03</f>
-        <v/>
-      </c>
-      <c r="I14" s="9">
-        <f>D14*0.0378</f>
-        <v/>
+      <c r="D14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="J14" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="9">
-        <f>G14+H14+I14+J14</f>
-        <v/>
-      </c>
-      <c r="L14" s="9">
-        <f>K14*0.05</f>
-        <v/>
-      </c>
-      <c r="M14" s="9">
-        <f>K14+L14</f>
-        <v/>
-      </c>
-      <c r="N14" s="9">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "May-2027")</f>
-        <v/>
-      </c>
-      <c r="O14" s="9">
-        <f>M14-N14</f>
-        <v/>
+      <c r="K14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -1330,52 +1263,43 @@
       <c r="C15" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="D15" s="5">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Jun-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E15" s="6">
-        <f>IF(C15&gt;0, D15/C15, 0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="4">
-        <f>IF(D15=0, "Not Started", IF(E15&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G15" s="5">
-        <f>IF(E15&gt;=0.99, D15*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H15" s="5">
-        <f>D15*0.03</f>
-        <v/>
-      </c>
-      <c r="I15" s="5">
-        <f>D15*0.0378</f>
-        <v/>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="5">
-        <f>G15+H15+I15+J15</f>
-        <v/>
-      </c>
-      <c r="L15" s="5">
-        <f>K15*0.05</f>
-        <v/>
-      </c>
-      <c r="M15" s="5">
-        <f>K15+L15</f>
-        <v/>
-      </c>
-      <c r="N15" s="5">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Jun-2027")</f>
-        <v/>
-      </c>
-      <c r="O15" s="5">
-        <f>M15-N15</f>
-        <v/>
+      <c r="K15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
@@ -1392,116 +1316,96 @@
       <c r="C16" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="D16" s="9">
-        <f>SUMIFS('Inward Bill Quick-Log'!G:G, 'Inward Bill Quick-Log'!E:E, "Jul-2027", 'Inward Bill Quick-Log'!C:C, "*Ajanta*")</f>
-        <v/>
-      </c>
-      <c r="E16" s="10">
-        <f>IF(C16&gt;0, D16/C16, 0)</f>
-        <v/>
-      </c>
-      <c r="F16" s="8">
-        <f>IF(D16=0, "Not Started", IF(E16&gt;=0.99, "Target Met", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G16" s="9">
-        <f>IF(E16&gt;=0.99, D16*0.03, 0)</f>
-        <v/>
-      </c>
-      <c r="H16" s="9">
-        <f>D16*0.03</f>
-        <v/>
-      </c>
-      <c r="I16" s="9">
-        <f>D16*0.0378</f>
-        <v/>
+      <c r="D16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="J16" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="9">
-        <f>G16+H16+I16+J16</f>
-        <v/>
-      </c>
-      <c r="L16" s="9">
-        <f>K16*0.05</f>
-        <v/>
-      </c>
-      <c r="M16" s="9">
-        <f>K16+L16</f>
-        <v/>
-      </c>
-      <c r="N16" s="9">
-        <f>SUMIFS('Ajanta Credit Notes Log'!G:G, 'Ajanta Credit Notes Log'!B:B, "Jul-2027")</f>
-        <v/>
-      </c>
-      <c r="O16" s="9">
-        <f>M16-N16</f>
-        <v/>
+      <c r="K16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>TOTAL / YTD</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>12 Months</t>
         </is>
       </c>
-      <c r="C17" s="12">
-        <f>SUM(C5:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="12">
-        <f>SUM(D5:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="13">
-        <f>IF(C17&gt;0, D17/C17, 0)</f>
-        <v/>
-      </c>
-      <c r="F17" s="11">
-        <f>IF(E17&gt;=0.99, "YTD Met", "Tracking")</f>
-        <v/>
-      </c>
-      <c r="G17" s="12">
-        <f>SUM(G5:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="12">
-        <f>SUM(H5:H16)</f>
-        <v/>
-      </c>
-      <c r="I17" s="12">
-        <f>SUM(I5:I16)</f>
-        <v/>
-      </c>
-      <c r="J17" s="12">
-        <f>SUM(J5:J16)</f>
-        <v/>
-      </c>
-      <c r="K17" s="12">
-        <f>SUM(K5:K16)</f>
-        <v/>
-      </c>
-      <c r="L17" s="12">
-        <f>SUM(L5:L16)</f>
-        <v/>
-      </c>
-      <c r="M17" s="12">
-        <f>SUM(M5:M16)</f>
-        <v/>
-      </c>
-      <c r="N17" s="12">
-        <f>SUM(N5:N16)</f>
-        <v/>
-      </c>
-      <c r="O17" s="12">
-        <f>SUM(O5:O16)</f>
-        <v/>
+      <c r="C17" s="13" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>2189453.1</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>0.18245</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>YTD Tracking</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>65683.59</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>65683.59</v>
+      </c>
+      <c r="I17" s="13" t="n">
+        <v>82761.33</v>
+      </c>
+      <c r="J17" s="13" t="n">
+        <v>54680.95</v>
+      </c>
+      <c r="K17" s="13" t="n">
+        <v>268809.46</v>
+      </c>
+      <c r="L17" s="13" t="n">
+        <v>13440.48</v>
+      </c>
+      <c r="M17" s="13" t="n">
+        <v>282249.94</v>
+      </c>
+      <c r="N17" s="13" t="n">
+        <v>198656.07</v>
+      </c>
+      <c r="O17" s="13" t="n">
+        <v>83593.87</v>
       </c>
     </row>
   </sheetData>
@@ -1527,7 +1431,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
@@ -1600,7 +1504,7 @@
           <t>Q2 (FY 26-27)</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Aug 2026 – Sep 2026 (2 Mo)</t>
         </is>
@@ -1608,28 +1512,25 @@
       <c r="C5" s="5" t="n">
         <v>2000000</v>
       </c>
-      <c r="D5" s="5">
-        <f>'Monthly Target Tracker'!D5+'Monthly Target Tracker'!D6</f>
-        <v/>
-      </c>
-      <c r="E5" s="6">
-        <f>IF(C5&gt;0, D5/C5, 0)</f>
-        <v/>
-      </c>
-      <c r="F5" s="4">
-        <f>IF(D5=0, "Pending", IF(E5&gt;=0.99, "Achieved", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G5" s="15" t="n">
+      <c r="D5" s="5" t="n">
+        <v>2189453.1</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>1.09473</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Achieved (109.5%)</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="H5" s="5">
-        <f>D5*G5</f>
-        <v/>
-      </c>
-      <c r="I5" s="5">
-        <f>H5*1.05</f>
-        <v/>
+      <c r="H5" s="5" t="n">
+        <v>43789.06</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>45978.51</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -1638,7 +1539,7 @@
           <t>Q3 (FY 26-27)</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Oct 2026 – Dec 2026 (3 Mo)</t>
         </is>
@@ -1646,28 +1547,25 @@
       <c r="C6" s="9" t="n">
         <v>3000000</v>
       </c>
-      <c r="D6" s="9">
-        <f>'Monthly Target Tracker'!D7+'Monthly Target Tracker'!D8+'Monthly Target Tracker'!D9</f>
-        <v/>
-      </c>
-      <c r="E6" s="10">
-        <f>IF(C6&gt;0, D6/C6, 0)</f>
-        <v/>
-      </c>
-      <c r="F6" s="8">
-        <f>IF(D6=0, "Pending", IF(E6&gt;=0.99, "Achieved", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G6" s="17" t="n">
+      <c r="D6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="n">
         <v>0.02</v>
       </c>
-      <c r="H6" s="9">
-        <f>D6*G6</f>
-        <v/>
-      </c>
-      <c r="I6" s="9">
-        <f>H6*1.05</f>
-        <v/>
+      <c r="H6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -1676,7 +1574,7 @@
           <t>Q4 (FY 26-27)</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Jan 2027 – Mar 2027 (3 Mo)</t>
         </is>
@@ -1684,28 +1582,25 @@
       <c r="C7" s="5" t="n">
         <v>3000000</v>
       </c>
-      <c r="D7" s="5">
-        <f>'Monthly Target Tracker'!D10+'Monthly Target Tracker'!D11+'Monthly Target Tracker'!D12</f>
-        <v/>
-      </c>
-      <c r="E7" s="6">
-        <f>IF(C7&gt;0, D7/C7, 0)</f>
-        <v/>
-      </c>
-      <c r="F7" s="4">
-        <f>IF(D7=0, "Pending", IF(E7&gt;=0.99, "Achieved", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G7" s="15" t="n">
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="H7" s="5">
-        <f>D7*G7</f>
-        <v/>
-      </c>
-      <c r="I7" s="5">
-        <f>H7*1.05</f>
-        <v/>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -1714,7 +1609,7 @@
           <t>Q1 (FY 27-28)</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Apr 2027 – Jul 2027 (4 Mo)</t>
         </is>
@@ -1722,69 +1617,62 @@
       <c r="C8" s="9" t="n">
         <v>4000000</v>
       </c>
-      <c r="D8" s="9">
-        <f>'Monthly Target Tracker'!D13+'Monthly Target Tracker'!D14+'Monthly Target Tracker'!D15+'Monthly Target Tracker'!D16</f>
-        <v/>
-      </c>
-      <c r="E8" s="10">
-        <f>IF(C8&gt;0, D8/C8, 0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="8">
-        <f>IF(D8=0, "Pending", IF(E8&gt;=0.99, "Achieved", "Shortfall"))</f>
-        <v/>
-      </c>
-      <c r="G8" s="17" t="n">
+      <c r="D8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="n">
         <v>0.02</v>
       </c>
-      <c r="H8" s="9">
-        <f>D8*G8</f>
-        <v/>
-      </c>
-      <c r="I8" s="9">
-        <f>H8*1.05</f>
-        <v/>
+      <c r="H8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>TOTAL QUARTERLY</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>12 Months Total</t>
         </is>
       </c>
-      <c r="C9" s="12">
-        <f>SUM(C5:C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="12">
-        <f>SUM(D5:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="13">
-        <f>IF(C9&gt;0, D9/C9, 0)</f>
-        <v/>
-      </c>
-      <c r="F9" s="11">
-        <f>IF(E9&gt;=0.99, "Target Met", "In Progress")</f>
-        <v/>
-      </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="C9" s="13" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>2189453.1</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>0.18245</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>2.00% Avg</t>
         </is>
       </c>
-      <c r="H9" s="12">
-        <f>SUM(H5:H8)</f>
-        <v/>
-      </c>
-      <c r="I9" s="12">
-        <f>SUM(I5:I8)</f>
-        <v/>
+      <c r="H9" s="13" t="n">
+        <v>43789.06</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>45978.51</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -1823,12 +1711,11 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>Sum of 12 Months Basic Purchases from Ajanta</t>
-        </is>
-      </c>
-      <c r="C13" s="26">
-        <f>D9</f>
-        <v/>
+          <t>Sum of Inward Basic Purchases from Ajanta (Aug + Sep)</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="n">
+        <v>2189453.1</v>
       </c>
       <c r="D13" s="27" t="n"/>
       <c r="E13" s="27" t="n"/>
@@ -1840,14 +1727,17 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>Annual Progress %</t>
-        </is>
-      </c>
-      <c r="B14" s="21">
-        <f>IF(C12&gt;0, C13/C12, 0)</f>
-        <v/>
-      </c>
-      <c r="C14" s="28" t="inlineStr"/>
+          <t>Annual Target Progress %</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>YTD Turnover / Annual Commitment</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="n">
+        <v>0.18245</v>
+      </c>
       <c r="D14" s="23" t="n"/>
       <c r="E14" s="23" t="n"/>
       <c r="F14" s="23" t="n"/>
@@ -1882,11 +1772,14 @@
           <t>Projected Annual ATB Payout (Basic)</t>
         </is>
       </c>
-      <c r="B16" s="21">
-        <f>C13*C15</f>
-        <v/>
-      </c>
-      <c r="C16" s="22" t="inlineStr"/>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>On Target Completion (3.00% on ₹1.20 Crore)</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="n">
+        <v>360000</v>
+      </c>
       <c r="D16" s="23" t="n"/>
       <c r="E16" s="23" t="n"/>
       <c r="F16" s="23" t="n"/>
@@ -1900,11 +1793,14 @@
           <t>Gross ATB with 5% IGST Credit Note</t>
         </is>
       </c>
-      <c r="B17" s="25">
-        <f>C16*1.05</f>
-        <v/>
-      </c>
-      <c r="C17" s="26" t="inlineStr"/>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>Full Credit Note Value Payable by Ajanta Shoes</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="n">
+        <v>378000</v>
+      </c>
       <c r="D17" s="27" t="n"/>
       <c r="E17" s="27" t="n"/>
       <c r="F17" s="27" t="n"/>
@@ -2025,12 +1921,12 @@
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>1900402723</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2045,18 +1941,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G5" s="31" t="n">
+      <c r="G5" s="5" t="n">
         <v>41332.56</v>
       </c>
-      <c r="H5" s="31" t="n">
+      <c r="H5" s="5" t="n">
         <v>2066.62</v>
       </c>
-      <c r="I5" s="31" t="n">
+      <c r="I5" s="5" t="n">
         <v>43399</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -2079,12 +1975,12 @@
       <c r="A6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>1900402722</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2099,18 +1995,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>Delight Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G6" s="32" t="n">
+      <c r="G6" s="9" t="n">
         <v>145384.32</v>
       </c>
-      <c r="H6" s="32" t="n">
+      <c r="H6" s="9" t="n">
         <v>7269.18</v>
       </c>
-      <c r="I6" s="32" t="n">
+      <c r="I6" s="9" t="n">
         <v>152653.5</v>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -2133,12 +2029,12 @@
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>1900402782</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2153,18 +2049,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G7" s="31" t="n">
+      <c r="G7" s="5" t="n">
         <v>59077.92</v>
       </c>
-      <c r="H7" s="31" t="n">
+      <c r="H7" s="5" t="n">
         <v>2953.88</v>
       </c>
-      <c r="I7" s="31" t="n">
+      <c r="I7" s="5" t="n">
         <v>62032</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -2187,12 +2083,12 @@
       <c r="A8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>1900402692</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2207,18 +2103,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G8" s="32" t="n">
+      <c r="G8" s="9" t="n">
         <v>49943.64</v>
       </c>
-      <c r="H8" s="32" t="n">
+      <c r="H8" s="9" t="n">
         <v>2497.16</v>
       </c>
-      <c r="I8" s="32" t="n">
+      <c r="I8" s="9" t="n">
         <v>52441</v>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -2241,12 +2137,12 @@
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>1900402693</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2261,18 +2157,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G9" s="31" t="n">
+      <c r="G9" s="5" t="n">
         <v>53376.3</v>
       </c>
-      <c r="H9" s="31" t="n">
+      <c r="H9" s="5" t="n">
         <v>2668.83</v>
       </c>
-      <c r="I9" s="31" t="n">
+      <c r="I9" s="5" t="n">
         <v>56045</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -2295,12 +2191,12 @@
       <c r="A10" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>1900402694</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2315,18 +2211,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G10" s="32" t="n">
+      <c r="G10" s="9" t="n">
         <v>5339.4</v>
       </c>
-      <c r="H10" s="32" t="n">
+      <c r="H10" s="9" t="n">
         <v>266.97</v>
       </c>
-      <c r="I10" s="32" t="n">
+      <c r="I10" s="9" t="n">
         <v>5606</v>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -2349,12 +2245,12 @@
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>1900402797</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2369,18 +2265,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G11" s="31" t="n">
+      <c r="G11" s="5" t="n">
         <v>80256.60000000001</v>
       </c>
-      <c r="H11" s="31" t="n">
+      <c r="H11" s="5" t="n">
         <v>4012.88</v>
       </c>
-      <c r="I11" s="31" t="n">
+      <c r="I11" s="5" t="n">
         <v>84269</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -2403,12 +2299,12 @@
       <c r="A12" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>1900402814</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2423,18 +2319,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G12" s="32" t="n">
+      <c r="G12" s="9" t="n">
         <v>6053.7</v>
       </c>
-      <c r="H12" s="32" t="n">
+      <c r="H12" s="9" t="n">
         <v>302.69</v>
       </c>
-      <c r="I12" s="32" t="n">
+      <c r="I12" s="9" t="n">
         <v>6356</v>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -2457,12 +2353,12 @@
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>1900402878</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2477,18 +2373,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G13" s="31" t="n">
+      <c r="G13" s="5" t="n">
         <v>16018.5</v>
       </c>
-      <c r="H13" s="31" t="n">
+      <c r="H13" s="5" t="n">
         <v>800.9299999999999</v>
       </c>
-      <c r="I13" s="31" t="n">
+      <c r="I13" s="5" t="n">
         <v>16819</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -2511,12 +2407,12 @@
       <c r="A14" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>1900402879</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2531,18 +2427,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G14" s="32" t="n">
+      <c r="G14" s="9" t="n">
         <v>38448</v>
       </c>
-      <c r="H14" s="32" t="n">
+      <c r="H14" s="9" t="n">
         <v>1922.42</v>
       </c>
-      <c r="I14" s="32" t="n">
+      <c r="I14" s="9" t="n">
         <v>40370</v>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -2565,12 +2461,12 @@
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>1900404091</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2585,18 +2481,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G15" s="31" t="n">
+      <c r="G15" s="5" t="n">
         <v>67615.32000000001</v>
       </c>
-      <c r="H15" s="31" t="n">
+      <c r="H15" s="5" t="n">
         <v>3380.79</v>
       </c>
-      <c r="I15" s="31" t="n">
+      <c r="I15" s="5" t="n">
         <v>70996</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -2619,12 +2515,12 @@
       <c r="A16" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>1900404102</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C16" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2639,18 +2535,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="F16" s="17" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G16" s="32" t="n">
+      <c r="G16" s="9" t="n">
         <v>26222.76</v>
       </c>
-      <c r="H16" s="32" t="n">
+      <c r="H16" s="9" t="n">
         <v>1311.15</v>
       </c>
-      <c r="I16" s="32" t="n">
+      <c r="I16" s="9" t="n">
         <v>27534</v>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -2673,12 +2569,12 @@
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>1900404784</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2693,18 +2589,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G17" s="31" t="n">
+      <c r="G17" s="5" t="n">
         <v>148593.96</v>
       </c>
-      <c r="H17" s="31" t="n">
+      <c r="H17" s="5" t="n">
         <v>7429.7</v>
       </c>
-      <c r="I17" s="31" t="n">
+      <c r="I17" s="5" t="n">
         <v>156024</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -2727,12 +2623,12 @@
       <c r="A18" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>1900404927</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2747,18 +2643,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G18" s="32" t="n">
+      <c r="G18" s="9" t="n">
         <v>65895.84</v>
       </c>
-      <c r="H18" s="32" t="n">
+      <c r="H18" s="9" t="n">
         <v>3294.76</v>
       </c>
-      <c r="I18" s="32" t="n">
+      <c r="I18" s="9" t="n">
         <v>69191</v>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -2781,12 +2677,12 @@
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>1900405148</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2801,18 +2697,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G19" s="31" t="n">
+      <c r="G19" s="5" t="n">
         <v>51158.7</v>
       </c>
-      <c r="H19" s="31" t="n">
+      <c r="H19" s="5" t="n">
         <v>2557.94</v>
       </c>
-      <c r="I19" s="31" t="n">
+      <c r="I19" s="5" t="n">
         <v>53717</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -2835,12 +2731,12 @@
       <c r="A20" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>1900405157</t>
         </is>
       </c>
-      <c r="C20" s="16" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2855,18 +2751,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F20" s="16" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G20" s="32" t="n">
+      <c r="G20" s="9" t="n">
         <v>21136.74</v>
       </c>
-      <c r="H20" s="32" t="n">
+      <c r="H20" s="9" t="n">
         <v>1056.85</v>
       </c>
-      <c r="I20" s="32" t="n">
+      <c r="I20" s="9" t="n">
         <v>22194</v>
       </c>
       <c r="J20" s="8" t="inlineStr">
@@ -2889,12 +2785,12 @@
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>1900405158</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2909,18 +2805,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G21" s="31" t="n">
+      <c r="G21" s="5" t="n">
         <v>32306.64</v>
       </c>
-      <c r="H21" s="31" t="n">
+      <c r="H21" s="5" t="n">
         <v>1615.33</v>
       </c>
-      <c r="I21" s="31" t="n">
+      <c r="I21" s="5" t="n">
         <v>33922</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2943,12 +2839,12 @@
       <c r="A22" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>1900405361</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -2963,18 +2859,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F22" s="16" t="inlineStr">
+      <c r="F22" s="17" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G22" s="32" t="n">
+      <c r="G22" s="9" t="n">
         <v>14040</v>
       </c>
-      <c r="H22" s="32" t="n">
+      <c r="H22" s="9" t="n">
         <v>702</v>
       </c>
-      <c r="I22" s="32" t="n">
+      <c r="I22" s="9" t="n">
         <v>14742</v>
       </c>
       <c r="J22" s="8" t="inlineStr">
@@ -2997,12 +2893,12 @@
       <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>1900405893</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3017,18 +2913,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G23" s="31" t="n">
+      <c r="G23" s="5" t="n">
         <v>71970.36</v>
       </c>
-      <c r="H23" s="31" t="n">
+      <c r="H23" s="5" t="n">
         <v>3598.53</v>
       </c>
-      <c r="I23" s="31" t="n">
+      <c r="I23" s="5" t="n">
         <v>75569</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -3051,12 +2947,12 @@
       <c r="A24" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>1900403625</t>
         </is>
       </c>
-      <c r="C24" s="16" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3071,18 +2967,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F24" s="16" t="inlineStr">
+      <c r="F24" s="17" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G24" s="32" t="n">
+      <c r="G24" s="9" t="n">
         <v>33098.4</v>
       </c>
-      <c r="H24" s="32" t="n">
+      <c r="H24" s="9" t="n">
         <v>1654.92</v>
       </c>
-      <c r="I24" s="32" t="n">
+      <c r="I24" s="9" t="n">
         <v>34753</v>
       </c>
       <c r="J24" s="8" t="inlineStr">
@@ -3105,12 +3001,12 @@
       <c r="A25" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>1900408353</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3125,18 +3021,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G25" s="31" t="n">
+      <c r="G25" s="5" t="n">
         <v>150038.88</v>
       </c>
-      <c r="H25" s="31" t="n">
+      <c r="H25" s="5" t="n">
         <v>7501.9</v>
       </c>
-      <c r="I25" s="31" t="n">
+      <c r="I25" s="5" t="n">
         <v>157541</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -3159,12 +3055,12 @@
       <c r="A26" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>1900408420</t>
         </is>
       </c>
-      <c r="C26" s="16" t="inlineStr">
+      <c r="C26" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3179,18 +3075,18 @@
           <t>Aug-2026</t>
         </is>
       </c>
-      <c r="F26" s="16" t="inlineStr">
+      <c r="F26" s="17" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G26" s="32" t="n">
+      <c r="G26" s="9" t="n">
         <v>14821.8</v>
       </c>
-      <c r="H26" s="32" t="n">
+      <c r="H26" s="9" t="n">
         <v>741.1</v>
       </c>
-      <c r="I26" s="32" t="n">
+      <c r="I26" s="9" t="n">
         <v>15563</v>
       </c>
       <c r="J26" s="8" t="inlineStr">
@@ -3213,12 +3109,12 @@
       <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>XPL/2041/26-27</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>XPANIA FOOTCARE LLP</t>
         </is>
@@ -3233,18 +3129,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F27" s="14" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
         <is>
           <t>M/s Sushila Boot House, Jharsuguda</t>
         </is>
       </c>
-      <c r="G27" s="31" t="n">
+      <c r="G27" s="5" t="n">
         <v>162196.34</v>
       </c>
-      <c r="H27" s="31" t="n">
+      <c r="H27" s="5" t="n">
         <v>8109.79</v>
       </c>
-      <c r="I27" s="31" t="n">
+      <c r="I27" s="5" t="n">
         <v>170306</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -3267,12 +3163,12 @@
       <c r="A28" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>1900410889</t>
         </is>
       </c>
-      <c r="C28" s="16" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3287,18 +3183,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="F28" s="17" t="inlineStr">
         <is>
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G28" s="32" t="n">
+      <c r="G28" s="9" t="n">
         <v>21803.52</v>
       </c>
-      <c r="H28" s="32" t="n">
+      <c r="H28" s="9" t="n">
         <v>1090.16</v>
       </c>
-      <c r="I28" s="32" t="n">
+      <c r="I28" s="9" t="n">
         <v>22894</v>
       </c>
       <c r="J28" s="8" t="inlineStr">
@@ -3321,12 +3217,12 @@
       <c r="A29" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>1900410928</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3341,18 +3237,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G29" s="31" t="n">
+      <c r="G29" s="5" t="n">
         <v>17959.08</v>
       </c>
-      <c r="H29" s="31" t="n">
+      <c r="H29" s="5" t="n">
         <v>897.95</v>
       </c>
-      <c r="I29" s="31" t="n">
+      <c r="I29" s="5" t="n">
         <v>18857</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -3375,12 +3271,12 @@
       <c r="A30" s="8" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>1900410970</t>
         </is>
       </c>
-      <c r="C30" s="16" t="inlineStr">
+      <c r="C30" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3395,18 +3291,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F30" s="16" t="inlineStr">
+      <c r="F30" s="17" t="inlineStr">
         <is>
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G30" s="32" t="n">
+      <c r="G30" s="9" t="n">
         <v>4036.2</v>
       </c>
-      <c r="H30" s="32" t="n">
+      <c r="H30" s="9" t="n">
         <v>201.81</v>
       </c>
-      <c r="I30" s="32" t="n">
+      <c r="I30" s="9" t="n">
         <v>4238</v>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -3429,12 +3325,12 @@
       <c r="A31" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>1900410890</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3449,18 +3345,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F31" s="14" t="inlineStr">
+      <c r="F31" s="15" t="inlineStr">
         <is>
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G31" s="31" t="n">
+      <c r="G31" s="5" t="n">
         <v>50893.44</v>
       </c>
-      <c r="H31" s="31" t="n">
+      <c r="H31" s="5" t="n">
         <v>2544.64</v>
       </c>
-      <c r="I31" s="31" t="n">
+      <c r="I31" s="5" t="n">
         <v>53438</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -3483,12 +3379,12 @@
       <c r="A32" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>1900410929</t>
         </is>
       </c>
-      <c r="C32" s="16" t="inlineStr">
+      <c r="C32" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3503,18 +3399,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F32" s="16" t="inlineStr">
+      <c r="F32" s="17" t="inlineStr">
         <is>
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G32" s="32" t="n">
+      <c r="G32" s="9" t="n">
         <v>54079.08</v>
       </c>
-      <c r="H32" s="32" t="n">
+      <c r="H32" s="9" t="n">
         <v>2703.93</v>
       </c>
-      <c r="I32" s="32" t="n">
+      <c r="I32" s="9" t="n">
         <v>56783</v>
       </c>
       <c r="J32" s="8" t="inlineStr">
@@ -3537,12 +3433,12 @@
       <c r="A33" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>1900410971</t>
         </is>
       </c>
-      <c r="C33" s="14" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3557,18 +3453,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F33" s="14" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G33" s="31" t="n">
+      <c r="G33" s="5" t="n">
         <v>32519.7</v>
       </c>
-      <c r="H33" s="31" t="n">
+      <c r="H33" s="5" t="n">
         <v>1626</v>
       </c>
-      <c r="I33" s="31" t="n">
+      <c r="I33" s="5" t="n">
         <v>34146</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -3591,12 +3487,12 @@
       <c r="A34" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>1900411104</t>
         </is>
       </c>
-      <c r="C34" s="16" t="inlineStr">
+      <c r="C34" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3611,18 +3507,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F34" s="16" t="inlineStr">
+      <c r="F34" s="17" t="inlineStr">
         <is>
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G34" s="32" t="n">
+      <c r="G34" s="9" t="n">
         <v>4393.2</v>
       </c>
-      <c r="H34" s="32" t="n">
+      <c r="H34" s="9" t="n">
         <v>219.66</v>
       </c>
-      <c r="I34" s="32" t="n">
+      <c r="I34" s="9" t="n">
         <v>4613</v>
       </c>
       <c r="J34" s="8" t="inlineStr">
@@ -3645,12 +3541,12 @@
       <c r="A35" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B35" s="15" t="inlineStr">
         <is>
           <t>1900412399</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr">
+      <c r="C35" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3665,18 +3561,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F35" s="14" t="inlineStr">
+      <c r="F35" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G35" s="31" t="n">
+      <c r="G35" s="5" t="n">
         <v>19989</v>
       </c>
-      <c r="H35" s="31" t="n">
+      <c r="H35" s="5" t="n">
         <v>999.45</v>
       </c>
-      <c r="I35" s="31" t="n">
+      <c r="I35" s="5" t="n">
         <v>20988</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3699,12 +3595,12 @@
       <c r="A36" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B36" s="17" t="inlineStr">
         <is>
           <t>1900412471</t>
         </is>
       </c>
-      <c r="C36" s="16" t="inlineStr">
+      <c r="C36" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3719,18 +3615,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F36" s="16" t="inlineStr">
+      <c r="F36" s="17" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G36" s="32" t="n">
+      <c r="G36" s="9" t="n">
         <v>11928.9</v>
       </c>
-      <c r="H36" s="32" t="n">
+      <c r="H36" s="9" t="n">
         <v>596.45</v>
       </c>
-      <c r="I36" s="32" t="n">
+      <c r="I36" s="9" t="n">
         <v>12525</v>
       </c>
       <c r="J36" s="8" t="inlineStr">
@@ -3753,12 +3649,12 @@
       <c r="A37" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B37" s="15" t="inlineStr">
         <is>
           <t>1900412530</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr">
+      <c r="C37" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3773,18 +3669,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F37" s="14" t="inlineStr">
+      <c r="F37" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G37" s="31" t="n">
+      <c r="G37" s="5" t="n">
         <v>11876.1</v>
       </c>
-      <c r="H37" s="31" t="n">
+      <c r="H37" s="5" t="n">
         <v>593.8099999999999</v>
       </c>
-      <c r="I37" s="31" t="n">
+      <c r="I37" s="5" t="n">
         <v>12470</v>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3807,12 +3703,12 @@
       <c r="A38" s="8" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="16" t="inlineStr">
+      <c r="B38" s="17" t="inlineStr">
         <is>
           <t>1900412536</t>
         </is>
       </c>
-      <c r="C38" s="16" t="inlineStr">
+      <c r="C38" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3827,18 +3723,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F38" s="16" t="inlineStr">
+      <c r="F38" s="17" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G38" s="32" t="n">
+      <c r="G38" s="9" t="n">
         <v>5696.7</v>
       </c>
-      <c r="H38" s="32" t="n">
+      <c r="H38" s="9" t="n">
         <v>284.84</v>
       </c>
-      <c r="I38" s="32" t="n">
+      <c r="I38" s="9" t="n">
         <v>5982</v>
       </c>
       <c r="J38" s="8" t="inlineStr">
@@ -3861,12 +3757,12 @@
       <c r="A39" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="15" t="inlineStr">
         <is>
           <t>XPL/2140/26-27</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr">
         <is>
           <t>XPANIA FOOTCARE LLP</t>
         </is>
@@ -3881,18 +3777,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F39" s="14" t="inlineStr">
+      <c r="F39" s="15" t="inlineStr">
         <is>
           <t>Mahavir Shoe House, Dhenkanal</t>
         </is>
       </c>
-      <c r="G39" s="31" t="n">
+      <c r="G39" s="5" t="n">
         <v>254563.8</v>
       </c>
-      <c r="H39" s="31" t="n">
+      <c r="H39" s="5" t="n">
         <v>12728.19</v>
       </c>
-      <c r="I39" s="31" t="n">
+      <c r="I39" s="5" t="n">
         <v>267292</v>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3915,12 +3811,12 @@
       <c r="A40" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>1900413999</t>
         </is>
       </c>
-      <c r="C40" s="16" t="inlineStr">
+      <c r="C40" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3935,18 +3831,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F40" s="16" t="inlineStr">
+      <c r="F40" s="17" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G40" s="32" t="n">
+      <c r="G40" s="9" t="n">
         <v>12386.16</v>
       </c>
-      <c r="H40" s="32" t="n">
+      <c r="H40" s="9" t="n">
         <v>619.3</v>
       </c>
-      <c r="I40" s="32" t="n">
+      <c r="I40" s="9" t="n">
         <v>13005</v>
       </c>
       <c r="J40" s="8" t="inlineStr">
@@ -3969,12 +3865,12 @@
       <c r="A41" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B41" s="15" t="inlineStr">
         <is>
           <t>1900414047</t>
         </is>
       </c>
-      <c r="C41" s="14" t="inlineStr">
+      <c r="C41" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -3989,18 +3885,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F41" s="14" t="inlineStr">
+      <c r="F41" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G41" s="31" t="n">
+      <c r="G41" s="5" t="n">
         <v>22786.2</v>
       </c>
-      <c r="H41" s="31" t="n">
+      <c r="H41" s="5" t="n">
         <v>1139.32</v>
       </c>
-      <c r="I41" s="31" t="n">
+      <c r="I41" s="5" t="n">
         <v>23926</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -4023,12 +3919,12 @@
       <c r="A42" s="8" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="16" t="inlineStr">
+      <c r="B42" s="17" t="inlineStr">
         <is>
           <t>1900415903</t>
         </is>
       </c>
-      <c r="C42" s="16" t="inlineStr">
+      <c r="C42" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4043,18 +3939,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F42" s="16" t="inlineStr">
+      <c r="F42" s="17" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G42" s="32" t="n">
+      <c r="G42" s="9" t="n">
         <v>9959.52</v>
       </c>
-      <c r="H42" s="32" t="n">
+      <c r="H42" s="9" t="n">
         <v>497.98</v>
       </c>
-      <c r="I42" s="32" t="n">
+      <c r="I42" s="9" t="n">
         <v>10458</v>
       </c>
       <c r="J42" s="8" t="inlineStr">
@@ -4077,12 +3973,12 @@
       <c r="A43" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B43" s="15" t="inlineStr">
         <is>
           <t>1900415994</t>
         </is>
       </c>
-      <c r="C43" s="14" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4097,18 +3993,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F43" s="14" t="inlineStr">
+      <c r="F43" s="15" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G43" s="31" t="n">
+      <c r="G43" s="5" t="n">
         <v>5339.4</v>
       </c>
-      <c r="H43" s="31" t="n">
+      <c r="H43" s="5" t="n">
         <v>266.97</v>
       </c>
-      <c r="I43" s="31" t="n">
+      <c r="I43" s="5" t="n">
         <v>5606</v>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -4131,12 +4027,12 @@
       <c r="A44" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="16" t="inlineStr">
+      <c r="B44" s="17" t="inlineStr">
         <is>
           <t>1900416575</t>
         </is>
       </c>
-      <c r="C44" s="16" t="inlineStr">
+      <c r="C44" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4151,18 +4047,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F44" s="16" t="inlineStr">
+      <c r="F44" s="17" t="inlineStr">
         <is>
           <t>Sri Sharvani Traders, Visakhapatnam</t>
         </is>
       </c>
-      <c r="G44" s="32" t="n">
+      <c r="G44" s="9" t="n">
         <v>287637.24</v>
       </c>
-      <c r="H44" s="32" t="n">
+      <c r="H44" s="9" t="n">
         <v>14381.87</v>
       </c>
-      <c r="I44" s="32" t="n">
+      <c r="I44" s="9" t="n">
         <v>302019</v>
       </c>
       <c r="J44" s="8" t="inlineStr">
@@ -4185,12 +4081,12 @@
       <c r="A45" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="14" t="inlineStr">
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>1900416574</t>
         </is>
       </c>
-      <c r="C45" s="14" t="inlineStr">
+      <c r="C45" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4205,18 +4101,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F45" s="14" t="inlineStr">
+      <c r="F45" s="15" t="inlineStr">
         <is>
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G45" s="31" t="n">
+      <c r="G45" s="5" t="n">
         <v>74536.92</v>
       </c>
-      <c r="H45" s="31" t="n">
+      <c r="H45" s="5" t="n">
         <v>3726.85</v>
       </c>
-      <c r="I45" s="31" t="n">
+      <c r="I45" s="5" t="n">
         <v>78264</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -4239,12 +4135,12 @@
       <c r="A46" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="16" t="inlineStr">
+      <c r="B46" s="17" t="inlineStr">
         <is>
           <t>1900416622</t>
         </is>
       </c>
-      <c r="C46" s="16" t="inlineStr">
+      <c r="C46" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4259,18 +4155,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F46" s="16" t="inlineStr">
+      <c r="F46" s="17" t="inlineStr">
         <is>
           <t>Sri Sharvani Traders, Visakhapatnam</t>
         </is>
       </c>
-      <c r="G46" s="32" t="n">
+      <c r="G46" s="9" t="n">
         <v>47888.16</v>
       </c>
-      <c r="H46" s="32" t="n">
+      <c r="H46" s="9" t="n">
         <v>2394.39</v>
       </c>
-      <c r="I46" s="32" t="n">
+      <c r="I46" s="9" t="n">
         <v>50283</v>
       </c>
       <c r="J46" s="8" t="inlineStr">
@@ -4293,12 +4189,12 @@
       <c r="A47" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B47" s="14" t="inlineStr">
+      <c r="B47" s="15" t="inlineStr">
         <is>
           <t>1900416634</t>
         </is>
       </c>
-      <c r="C47" s="14" t="inlineStr">
+      <c r="C47" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4313,18 +4209,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F47" s="14" t="inlineStr">
+      <c r="F47" s="15" t="inlineStr">
         <is>
           <t>Sri Sharvani Traders, Visakhapatnam</t>
         </is>
       </c>
-      <c r="G47" s="31" t="n">
+      <c r="G47" s="5" t="n">
         <v>37721.64</v>
       </c>
-      <c r="H47" s="31" t="n">
+      <c r="H47" s="5" t="n">
         <v>1886.09</v>
       </c>
-      <c r="I47" s="31" t="n">
+      <c r="I47" s="5" t="n">
         <v>39608</v>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -4347,12 +4243,12 @@
       <c r="A48" s="8" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="16" t="inlineStr">
+      <c r="B48" s="17" t="inlineStr">
         <is>
           <t>1900416912</t>
         </is>
       </c>
-      <c r="C48" s="16" t="inlineStr">
+      <c r="C48" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4367,18 +4263,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F48" s="16" t="inlineStr">
+      <c r="F48" s="17" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G48" s="32" t="n">
+      <c r="G48" s="9" t="n">
         <v>36525.72</v>
       </c>
-      <c r="H48" s="32" t="n">
+      <c r="H48" s="9" t="n">
         <v>1826.27</v>
       </c>
-      <c r="I48" s="32" t="n">
+      <c r="I48" s="9" t="n">
         <v>38352</v>
       </c>
       <c r="J48" s="8" t="inlineStr">
@@ -4401,12 +4297,12 @@
       <c r="A49" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="14" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>1900416927</t>
         </is>
       </c>
-      <c r="C49" s="14" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4421,18 +4317,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F49" s="14" t="inlineStr">
+      <c r="F49" s="15" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G49" s="31" t="n">
+      <c r="G49" s="5" t="n">
         <v>23500.2</v>
       </c>
-      <c r="H49" s="31" t="n">
+      <c r="H49" s="5" t="n">
         <v>1175.02</v>
       </c>
-      <c r="I49" s="31" t="n">
+      <c r="I49" s="5" t="n">
         <v>24675</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -4455,12 +4351,12 @@
       <c r="A50" s="8" t="n">
         <v>46</v>
       </c>
-      <c r="B50" s="16" t="inlineStr">
+      <c r="B50" s="17" t="inlineStr">
         <is>
           <t>1900416947</t>
         </is>
       </c>
-      <c r="C50" s="16" t="inlineStr">
+      <c r="C50" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4475,18 +4371,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F50" s="16" t="inlineStr">
+      <c r="F50" s="17" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G50" s="32" t="n">
+      <c r="G50" s="9" t="n">
         <v>23139.18</v>
       </c>
-      <c r="H50" s="32" t="n">
+      <c r="H50" s="9" t="n">
         <v>1156.96</v>
       </c>
-      <c r="I50" s="32" t="n">
+      <c r="I50" s="9" t="n">
         <v>24296</v>
       </c>
       <c r="J50" s="8" t="inlineStr">
@@ -4509,12 +4405,12 @@
       <c r="A51" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B51" s="14" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>1900417275</t>
         </is>
       </c>
-      <c r="C51" s="14" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4529,18 +4425,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F51" s="14" t="inlineStr">
+      <c r="F51" s="15" t="inlineStr">
         <is>
           <t>Sri Sharvani Traders, Visakhapatnam</t>
         </is>
       </c>
-      <c r="G51" s="31" t="n">
+      <c r="G51" s="5" t="n">
         <v>41721.6</v>
       </c>
-      <c r="H51" s="31" t="n">
+      <c r="H51" s="5" t="n">
         <v>2086.08</v>
       </c>
-      <c r="I51" s="31" t="n">
+      <c r="I51" s="5" t="n">
         <v>43808</v>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -4563,12 +4459,12 @@
       <c r="A52" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="16" t="inlineStr">
+      <c r="B52" s="17" t="inlineStr">
         <is>
           <t>1900417852</t>
         </is>
       </c>
-      <c r="C52" s="16" t="inlineStr">
+      <c r="C52" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4583,18 +4479,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F52" s="16" t="inlineStr">
+      <c r="F52" s="17" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Malkangiri</t>
         </is>
       </c>
-      <c r="G52" s="32" t="n">
+      <c r="G52" s="9" t="n">
         <v>26716.8</v>
       </c>
-      <c r="H52" s="32" t="n">
+      <c r="H52" s="9" t="n">
         <v>1335.84</v>
       </c>
-      <c r="I52" s="32" t="n">
+      <c r="I52" s="9" t="n">
         <v>28053</v>
       </c>
       <c r="J52" s="8" t="inlineStr">
@@ -4617,12 +4513,12 @@
       <c r="A53" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="B53" s="14" t="inlineStr">
+      <c r="B53" s="15" t="inlineStr">
         <is>
           <t>1900417853</t>
         </is>
       </c>
-      <c r="C53" s="14" t="inlineStr">
+      <c r="C53" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4637,18 +4533,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F53" s="14" t="inlineStr">
+      <c r="F53" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G53" s="31" t="n">
+      <c r="G53" s="5" t="n">
         <v>8283.120000000001</v>
       </c>
-      <c r="H53" s="31" t="n">
+      <c r="H53" s="5" t="n">
         <v>414.15</v>
       </c>
-      <c r="I53" s="31" t="n">
+      <c r="I53" s="5" t="n">
         <v>8697</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -4671,12 +4567,12 @@
       <c r="A54" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="16" t="inlineStr">
+      <c r="B54" s="17" t="inlineStr">
         <is>
           <t>1900417888</t>
         </is>
       </c>
-      <c r="C54" s="16" t="inlineStr">
+      <c r="C54" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4691,18 +4587,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F54" s="16" t="inlineStr">
+      <c r="F54" s="17" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Malkangiri</t>
         </is>
       </c>
-      <c r="G54" s="32" t="n">
+      <c r="G54" s="9" t="n">
         <v>5696.7</v>
       </c>
-      <c r="H54" s="32" t="n">
+      <c r="H54" s="9" t="n">
         <v>284.84</v>
       </c>
-      <c r="I54" s="32" t="n">
+      <c r="I54" s="9" t="n">
         <v>5982</v>
       </c>
       <c r="J54" s="8" t="inlineStr">
@@ -4725,12 +4621,12 @@
       <c r="A55" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="B55" s="14" t="inlineStr">
+      <c r="B55" s="15" t="inlineStr">
         <is>
           <t>1900417889</t>
         </is>
       </c>
-      <c r="C55" s="14" t="inlineStr">
+      <c r="C55" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4745,18 +4641,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F55" s="14" t="inlineStr">
+      <c r="F55" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G55" s="31" t="n">
+      <c r="G55" s="5" t="n">
         <v>14875.8</v>
       </c>
-      <c r="H55" s="31" t="n">
+      <c r="H55" s="5" t="n">
         <v>743.8</v>
       </c>
-      <c r="I55" s="31" t="n">
+      <c r="I55" s="5" t="n">
         <v>15620</v>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -4779,12 +4675,12 @@
       <c r="A56" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="B56" s="16" t="inlineStr">
+      <c r="B56" s="17" t="inlineStr">
         <is>
           <t>1900417925</t>
         </is>
       </c>
-      <c r="C56" s="16" t="inlineStr">
+      <c r="C56" s="17" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4799,18 +4695,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F56" s="16" t="inlineStr">
+      <c r="F56" s="17" t="inlineStr">
         <is>
           <t>M/s Sri Brundabana Enterprises, Malkangiri</t>
         </is>
       </c>
-      <c r="G56" s="32" t="n">
+      <c r="G56" s="9" t="n">
         <v>61896.78</v>
       </c>
-      <c r="H56" s="32" t="n">
+      <c r="H56" s="9" t="n">
         <v>3094.85</v>
       </c>
-      <c r="I56" s="32" t="n">
+      <c r="I56" s="9" t="n">
         <v>64992</v>
       </c>
       <c r="J56" s="8" t="inlineStr">
@@ -4833,12 +4729,12 @@
       <c r="A57" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="B57" s="14" t="inlineStr">
+      <c r="B57" s="15" t="inlineStr">
         <is>
           <t>1900417926</t>
         </is>
       </c>
-      <c r="C57" s="14" t="inlineStr">
+      <c r="C57" s="15" t="inlineStr">
         <is>
           <t>Ajanta Shoes India Pvt. Ltd.</t>
         </is>
@@ -4853,18 +4749,18 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="F57" s="14" t="inlineStr">
+      <c r="F57" s="15" t="inlineStr">
         <is>
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G57" s="31" t="n">
+      <c r="G57" s="5" t="n">
         <v>21536.7</v>
       </c>
-      <c r="H57" s="31" t="n">
+      <c r="H57" s="5" t="n">
         <v>1076.84</v>
       </c>
-      <c r="I57" s="31" t="n">
+      <c r="I57" s="5" t="n">
         <v>22614</v>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -4887,12 +4783,12 @@
       <c r="A58" s="8" t="n">
         <v>54</v>
       </c>
-      <c r="B58" s="16" t="inlineStr">
+      <c r="B58" s="17" t="inlineStr">
         <is>
           <t>XPL/2327/26-27</t>
         </is>
       </c>
-      <c r="C58" s="16" t="inlineStr">
+      <c r="C58" s="17" t="inlineStr">
         <is>
           <t>XPANIA FOOTCARE LLP</t>
         </is>
@@ -4907,18 +4803,18 @@
           <t>Oct-2026</t>
         </is>
       </c>
-      <c r="F58" s="16" t="inlineStr">
+      <c r="F58" s="17" t="inlineStr">
         <is>
           <t>Mahavir Shoe House, Dhenkanal</t>
         </is>
       </c>
-      <c r="G58" s="32" t="n">
+      <c r="G58" s="9" t="n">
         <v>134953.2</v>
       </c>
-      <c r="H58" s="32" t="n">
+      <c r="H58" s="9" t="n">
         <v>6747.66</v>
       </c>
-      <c r="I58" s="32" t="n">
+      <c r="I58" s="9" t="n">
         <v>141701</v>
       </c>
       <c r="J58" s="8" t="inlineStr">
@@ -4941,12 +4837,12 @@
       <c r="A59" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="B59" s="14" t="inlineStr">
+      <c r="B59" s="15" t="inlineStr">
         <is>
           <t>XPL/2367/26-27</t>
         </is>
       </c>
-      <c r="C59" s="14" t="inlineStr">
+      <c r="C59" s="15" t="inlineStr">
         <is>
           <t>XPANIA FOOTCARE LLP</t>
         </is>
@@ -4961,18 +4857,18 @@
           <t>Oct-2026</t>
         </is>
       </c>
-      <c r="F59" s="14" t="inlineStr">
+      <c r="F59" s="15" t="inlineStr">
         <is>
           <t>SHREE ADITYA FOOT FASHION</t>
         </is>
       </c>
-      <c r="G59" s="31" t="n">
+      <c r="G59" s="5" t="n">
         <v>105402</v>
       </c>
-      <c r="H59" s="31" t="n">
+      <c r="H59" s="5" t="n">
         <v>5270.1</v>
       </c>
-      <c r="I59" s="31" t="n">
+      <c r="I59" s="5" t="n">
         <v>110672</v>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -4995,12 +4891,12 @@
       <c r="A60" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="B60" s="16" t="inlineStr">
+      <c r="B60" s="17" t="inlineStr">
         <is>
           <t>XPL/2366/26-27</t>
         </is>
       </c>
-      <c r="C60" s="16" t="inlineStr">
+      <c r="C60" s="17" t="inlineStr">
         <is>
           <t>XPANIA FOOTCARE LLP</t>
         </is>
@@ -5015,18 +4911,18 @@
           <t>Oct-2026</t>
         </is>
       </c>
-      <c r="F60" s="16" t="inlineStr">
+      <c r="F60" s="17" t="inlineStr">
         <is>
           <t>M/S. RAJAN TRADERS</t>
         </is>
       </c>
-      <c r="G60" s="32" t="n">
+      <c r="G60" s="9" t="n">
         <v>104874</v>
       </c>
-      <c r="H60" s="32" t="n">
+      <c r="H60" s="9" t="n">
         <v>5243.7</v>
       </c>
-      <c r="I60" s="32" t="n">
+      <c r="I60" s="9" t="n">
         <v>110118</v>
       </c>
       <c r="J60" s="8" t="inlineStr">
@@ -5049,12 +4945,12 @@
       <c r="A61" s="4" t="n">
         <v>57</v>
       </c>
-      <c r="B61" s="14" t="inlineStr">
+      <c r="B61" s="15" t="inlineStr">
         <is>
           <t>XPL/2369/26-27</t>
         </is>
       </c>
-      <c r="C61" s="14" t="inlineStr">
+      <c r="C61" s="15" t="inlineStr">
         <is>
           <t>XPANIA FOOTCARE LLP</t>
         </is>
@@ -5069,18 +4965,18 @@
           <t>Oct-2026</t>
         </is>
       </c>
-      <c r="F61" s="14" t="inlineStr">
+      <c r="F61" s="15" t="inlineStr">
         <is>
           <t>SHREE ADITYA FOOT FASHION</t>
         </is>
       </c>
-      <c r="G61" s="31" t="n">
+      <c r="G61" s="5" t="n">
         <v>13752</v>
       </c>
-      <c r="H61" s="31" t="n">
+      <c r="H61" s="5" t="n">
         <v>687.6</v>
       </c>
-      <c r="I61" s="31" t="n">
+      <c r="I61" s="5" t="n">
         <v>14440</v>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -5100,39 +4996,36 @@
       </c>
     </row>
     <row r="62" ht="24" customHeight="1">
-      <c r="A62" s="11" t="inlineStr">
+      <c r="A62" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B62" s="11" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>57 Bills</t>
         </is>
       </c>
-      <c r="C62" s="33" t="n"/>
-      <c r="D62" s="33" t="n"/>
-      <c r="E62" s="33" t="n"/>
-      <c r="F62" s="33" t="n"/>
-      <c r="G62" s="12">
-        <f>SUM(G5:G61)</f>
-        <v/>
-      </c>
-      <c r="H62" s="12">
-        <f>SUM(H5:H61)</f>
-        <v/>
-      </c>
-      <c r="I62" s="12">
-        <f>SUM(I5:I61)</f>
-        <v/>
-      </c>
-      <c r="J62" s="11" t="inlineStr">
+      <c r="C62" s="31" t="n"/>
+      <c r="D62" s="31" t="n"/>
+      <c r="E62" s="31" t="n"/>
+      <c r="F62" s="31" t="n"/>
+      <c r="G62" s="32" t="n">
+        <v>2965194.44</v>
+      </c>
+      <c r="H62" s="32" t="n">
+        <v>148259.69</v>
+      </c>
+      <c r="I62" s="32" t="n">
+        <v>3113457.5</v>
+      </c>
+      <c r="J62" s="12" t="inlineStr">
         <is>
           <t>100% VERIFIED</t>
         </is>
       </c>
-      <c r="K62" s="33" t="n"/>
-      <c r="L62" s="33" t="n"/>
+      <c r="K62" s="31" t="n"/>
+      <c r="L62" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5251,13 +5144,13 @@
           <t>3.78% Retail Scheme (August 2026 Purchases)</t>
         </is>
       </c>
-      <c r="E5" s="31" t="n">
+      <c r="E5" s="5" t="n">
         <v>43710.48</v>
       </c>
-      <c r="F5" s="31" t="n">
+      <c r="F5" s="5" t="n">
         <v>2185.52</v>
       </c>
-      <c r="G5" s="31" t="n">
+      <c r="G5" s="5" t="n">
         <v>45896</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -5297,13 +5190,13 @@
           <t>3.00% Cash Discount (August Prompt Settlement)</t>
         </is>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="E6" s="9" t="n">
         <v>35763.92</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="9" t="n">
         <v>1788.2</v>
       </c>
-      <c r="G6" s="32" t="n">
+      <c r="G6" s="9" t="n">
         <v>37552.12</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -5343,13 +5236,13 @@
           <t>Rate Difference Rebate (UL 979E/CH+M Settlement)</t>
         </is>
       </c>
-      <c r="E7" s="31" t="n">
+      <c r="E7" s="5" t="n">
         <v>2641.86</v>
       </c>
-      <c r="F7" s="31" t="n">
+      <c r="F7" s="5" t="n">
         <v>132.09</v>
       </c>
-      <c r="G7" s="31" t="n">
+      <c r="G7" s="5" t="n">
         <v>2773.95</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -5389,13 +5282,13 @@
           <t>Non-Bengal Scratch Coupon Scheme (Aug Promo)</t>
         </is>
       </c>
-      <c r="E8" s="32" t="n">
+      <c r="E8" s="9" t="n">
         <v>24501.9</v>
       </c>
-      <c r="F8" s="32" t="n">
+      <c r="F8" s="9" t="n">
         <v>1225.1</v>
       </c>
-      <c r="G8" s="32" t="n">
+      <c r="G8" s="9" t="n">
         <v>25727</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -5435,13 +5328,13 @@
           <t>2.00% QTB / Cash Discount (Sep 2026 Settlement)</t>
         </is>
       </c>
-      <c r="E9" s="31" t="n">
+      <c r="E9" s="5" t="n">
         <v>19945.71</v>
       </c>
-      <c r="F9" s="31" t="n">
+      <c r="F9" s="5" t="n">
         <v>997.29</v>
       </c>
-      <c r="G9" s="31" t="n">
+      <c r="G9" s="5" t="n">
         <v>20943</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -5481,13 +5374,13 @@
           <t>Slab Scheme Bonus (Sep New State Target Bonus)</t>
         </is>
       </c>
-      <c r="E10" s="32" t="n">
+      <c r="E10" s="9" t="n">
         <v>24933.33</v>
       </c>
-      <c r="F10" s="32" t="n">
+      <c r="F10" s="9" t="n">
         <v>1246.67</v>
       </c>
-      <c r="G10" s="32" t="n">
+      <c r="G10" s="9" t="n">
         <v>26180</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -5527,13 +5420,13 @@
           <t>3.78% Retail Scheme (September 2026 Purchases)</t>
         </is>
       </c>
-      <c r="E11" s="31" t="n">
+      <c r="E11" s="5" t="n">
         <v>37699.05</v>
       </c>
-      <c r="F11" s="31" t="n">
+      <c r="F11" s="5" t="n">
         <v>1884.95</v>
       </c>
-      <c r="G11" s="31" t="n">
+      <c r="G11" s="5" t="n">
         <v>39584</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -5553,33 +5446,30 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>7 Notes</t>
         </is>
       </c>
-      <c r="C12" s="33" t="n"/>
-      <c r="D12" s="33" t="n"/>
-      <c r="E12" s="12">
-        <f>SUM(E5:E11)</f>
-        <v/>
-      </c>
-      <c r="F12" s="12">
-        <f>SUM(F5:F11)</f>
-        <v/>
-      </c>
-      <c r="G12" s="12">
-        <f>SUM(G5:G11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="33" t="n"/>
-      <c r="I12" s="33" t="n"/>
-      <c r="J12" s="11" t="inlineStr">
+      <c r="C12" s="31" t="n"/>
+      <c r="D12" s="31" t="n"/>
+      <c r="E12" s="32" t="n">
+        <v>189196.25</v>
+      </c>
+      <c r="F12" s="32" t="n">
+        <v>9459.82</v>
+      </c>
+      <c r="G12" s="32" t="n">
+        <v>198656.07</v>
+      </c>
+      <c r="H12" s="31" t="n"/>
+      <c r="I12" s="31" t="n"/>
+      <c r="J12" s="12" t="inlineStr">
         <is>
           <t>100% MATCH</t>
         </is>

</xml_diff>

<commit_message>
Fix number formatting from custom Rupee symbol to standard Excel format for Chrome and web viewer compatibility
</commit_message>
<xml_diff>
--- a/Ajanta_Target_and_Scheme_Tracker_FY26-27.xlsx
+++ b/Ajanta_Target_and_Scheme_Tracker_FY26-27.xlsx
@@ -163,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -243,6 +243,22 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -642,6 +658,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -730,10 +747,10 @@
           <t>Q2</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="33" t="n">
         <v>1000000</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="33" t="n">
         <v>1192130.34</v>
       </c>
       <c r="E5" s="6" t="n">
@@ -744,31 +761,31 @@
           <t>Target Met</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="33" t="n">
         <v>35763.91</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="33" t="n">
         <v>35763.91</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="33" t="n">
         <v>45062.53</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J5" s="33" t="n">
         <v>28500.95</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K5" s="33" t="n">
         <v>145091.3</v>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="L5" s="33" t="n">
         <v>7254.57</v>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="M5" s="33" t="n">
         <v>152345.87</v>
       </c>
-      <c r="N5" s="5" t="n">
+      <c r="N5" s="33" t="n">
         <v>111949.07</v>
       </c>
-      <c r="O5" s="5" t="n">
+      <c r="O5" s="33" t="n">
         <v>40396.8</v>
       </c>
     </row>
@@ -783,10 +800,10 @@
           <t>Q2</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="34" t="n">
         <v>1000000</v>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="34" t="n">
         <v>997322.76</v>
       </c>
       <c r="E6" s="10" t="n">
@@ -797,31 +814,31 @@
           <t>Target Met</t>
         </is>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="34" t="n">
         <v>29919.68</v>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="H6" s="34" t="n">
         <v>29919.68</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="I6" s="34" t="n">
         <v>37698.8</v>
       </c>
-      <c r="J6" s="9" t="n">
+      <c r="J6" s="34" t="n">
         <v>26180</v>
       </c>
-      <c r="K6" s="9" t="n">
+      <c r="K6" s="34" t="n">
         <v>123718.16</v>
       </c>
-      <c r="L6" s="9" t="n">
+      <c r="L6" s="34" t="n">
         <v>6185.91</v>
       </c>
-      <c r="M6" s="9" t="n">
+      <c r="M6" s="34" t="n">
         <v>129904.07</v>
       </c>
-      <c r="N6" s="9" t="n">
+      <c r="N6" s="34" t="n">
         <v>86707</v>
       </c>
-      <c r="O6" s="9" t="n">
+      <c r="O6" s="34" t="n">
         <v>43197.07</v>
       </c>
     </row>
@@ -836,10 +853,10 @@
           <t>Q3</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="33" t="n">
         <v>1000000</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="33" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="6" t="n">
@@ -850,31 +867,31 @@
           <t>Pending Invoices</t>
         </is>
       </c>
-      <c r="G7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="5" t="n">
+      <c r="G7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -889,10 +906,10 @@
           <t>Q3</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="34" t="n">
         <v>1000000</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="34" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="n">
@@ -903,31 +920,31 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="9" t="n">
+      <c r="G8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -942,10 +959,10 @@
           <t>Q3</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="33" t="n">
         <v>1000000</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="33" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="6" t="n">
@@ -956,31 +973,31 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="5" t="n">
+      <c r="G9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -995,10 +1012,10 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="34" t="n">
         <v>1000000</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="34" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="10" t="n">
@@ -1009,31 +1026,31 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="9" t="n">
+      <c r="G10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1048,10 +1065,10 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="33" t="n">
         <v>1000000</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="33" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="6" t="n">
@@ -1062,31 +1079,31 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="5" t="n">
+      <c r="G11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1101,10 +1118,10 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="34" t="n">
         <v>1000000</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="34" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="10" t="n">
@@ -1115,31 +1132,31 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="9" t="n">
+      <c r="G12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1154,10 +1171,10 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="33" t="n">
         <v>1000000</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="33" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
@@ -1168,31 +1185,31 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="5" t="n">
+      <c r="G13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1207,10 +1224,10 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="34" t="n">
         <v>1000000</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="34" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="n">
@@ -1221,31 +1238,31 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="9" t="n">
+      <c r="G14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1260,10 +1277,10 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="33" t="n">
         <v>1000000</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="33" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="6" t="n">
@@ -1274,31 +1291,31 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="5" t="n">
+      <c r="G15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1313,10 +1330,10 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="34" t="n">
         <v>1000000</v>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="34" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="10" t="n">
@@ -1327,31 +1344,31 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="9" t="n">
+      <c r="G16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1366,10 +1383,10 @@
           <t>12 Months</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="35" t="n">
         <v>12000000</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="35" t="n">
         <v>2189453.1</v>
       </c>
       <c r="E17" s="14" t="n">
@@ -1380,31 +1397,31 @@
           <t>YTD Tracking</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
+      <c r="G17" s="35" t="n">
         <v>65683.59</v>
       </c>
-      <c r="H17" s="13" t="n">
+      <c r="H17" s="35" t="n">
         <v>65683.59</v>
       </c>
-      <c r="I17" s="13" t="n">
+      <c r="I17" s="35" t="n">
         <v>82761.33</v>
       </c>
-      <c r="J17" s="13" t="n">
+      <c r="J17" s="35" t="n">
         <v>54680.95</v>
       </c>
-      <c r="K17" s="13" t="n">
+      <c r="K17" s="35" t="n">
         <v>268809.46</v>
       </c>
-      <c r="L17" s="13" t="n">
+      <c r="L17" s="35" t="n">
         <v>13440.48</v>
       </c>
-      <c r="M17" s="13" t="n">
+      <c r="M17" s="35" t="n">
         <v>282249.94</v>
       </c>
-      <c r="N17" s="13" t="n">
+      <c r="N17" s="35" t="n">
         <v>198656.07</v>
       </c>
-      <c r="O17" s="13" t="n">
+      <c r="O17" s="35" t="n">
         <v>83593.87</v>
       </c>
     </row>
@@ -1451,6 +1468,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1509,10 +1527,10 @@
           <t>Aug 2026 – Sep 2026 (2 Mo)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="33" t="n">
         <v>2000000</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="33" t="n">
         <v>2189453.1</v>
       </c>
       <c r="E5" s="6" t="n">
@@ -1526,10 +1544,10 @@
       <c r="G5" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="33" t="n">
         <v>43789.06</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="33" t="n">
         <v>45978.51</v>
       </c>
     </row>
@@ -1544,10 +1562,10 @@
           <t>Oct 2026 – Dec 2026 (3 Mo)</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="34" t="n">
         <v>3000000</v>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="34" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="10" t="n">
@@ -1561,10 +1579,10 @@
       <c r="G6" s="18" t="n">
         <v>0.02</v>
       </c>
-      <c r="H6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="9" t="n">
+      <c r="H6" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1579,10 +1597,10 @@
           <t>Jan 2027 – Mar 2027 (3 Mo)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="33" t="n">
         <v>3000000</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="33" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="6" t="n">
@@ -1596,10 +1614,10 @@
       <c r="G7" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="H7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="5" t="n">
+      <c r="H7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1614,10 +1632,10 @@
           <t>Apr 2027 – Jul 2027 (4 Mo)</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="34" t="n">
         <v>4000000</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="34" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="n">
@@ -1631,10 +1649,10 @@
       <c r="G8" s="18" t="n">
         <v>0.02</v>
       </c>
-      <c r="H8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="9" t="n">
+      <c r="H8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1649,10 +1667,10 @@
           <t>12 Months Total</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="35" t="n">
         <v>12000000</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="35" t="n">
         <v>2189453.1</v>
       </c>
       <c r="E9" s="14" t="n">
@@ -1668,13 +1686,14 @@
           <t>2.00% Avg</t>
         </is>
       </c>
-      <c r="H9" s="13" t="n">
+      <c r="H9" s="35" t="n">
         <v>43789.06</v>
       </c>
-      <c r="I9" s="13" t="n">
+      <c r="I9" s="35" t="n">
         <v>45978.51</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
@@ -1693,7 +1712,7 @@
           <t>Contract Section 2.0 (Aug 2026 to Jul 2027)</t>
         </is>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="36" t="n">
         <v>12000000</v>
       </c>
       <c r="D12" s="23" t="n"/>
@@ -1714,7 +1733,7 @@
           <t>Sum of Inward Basic Purchases from Ajanta (Aug + Sep)</t>
         </is>
       </c>
-      <c r="C13" s="26" t="n">
+      <c r="C13" s="37" t="n">
         <v>2189453.1</v>
       </c>
       <c r="D13" s="27" t="n"/>
@@ -1777,7 +1796,7 @@
           <t>On Target Completion (3.00% on ₹1.20 Crore)</t>
         </is>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="36" t="n">
         <v>360000</v>
       </c>
       <c r="D16" s="23" t="n"/>
@@ -1798,7 +1817,7 @@
           <t>Full Credit Note Value Payable by Ajanta Shoes</t>
         </is>
       </c>
-      <c r="C17" s="26" t="n">
+      <c r="C17" s="37" t="n">
         <v>378000</v>
       </c>
       <c r="D17" s="27" t="n"/>
@@ -1855,6 +1874,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="30" t="inlineStr">
         <is>
@@ -1946,13 +1966,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="33" t="n">
         <v>41332.56</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="33" t="n">
         <v>2066.62</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="33" t="n">
         <v>43399</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -2000,13 +2020,13 @@
           <t>Delight Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="34" t="n">
         <v>145384.32</v>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="H6" s="34" t="n">
         <v>7269.18</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="I6" s="34" t="n">
         <v>152653.5</v>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -2054,13 +2074,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="33" t="n">
         <v>59077.92</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="33" t="n">
         <v>2953.88</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="I7" s="33" t="n">
         <v>62032</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -2108,13 +2128,13 @@
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="34" t="n">
         <v>49943.64</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="H8" s="34" t="n">
         <v>2497.16</v>
       </c>
-      <c r="I8" s="9" t="n">
+      <c r="I8" s="34" t="n">
         <v>52441</v>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -2162,13 +2182,13 @@
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="33" t="n">
         <v>53376.3</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="33" t="n">
         <v>2668.83</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="I9" s="33" t="n">
         <v>56045</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -2216,13 +2236,13 @@
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G10" s="34" t="n">
         <v>5339.4</v>
       </c>
-      <c r="H10" s="9" t="n">
+      <c r="H10" s="34" t="n">
         <v>266.97</v>
       </c>
-      <c r="I10" s="9" t="n">
+      <c r="I10" s="34" t="n">
         <v>5606</v>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -2270,13 +2290,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="33" t="n">
         <v>80256.60000000001</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="33" t="n">
         <v>4012.88</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="I11" s="33" t="n">
         <v>84269</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -2324,13 +2344,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G12" s="34" t="n">
         <v>6053.7</v>
       </c>
-      <c r="H12" s="9" t="n">
+      <c r="H12" s="34" t="n">
         <v>302.69</v>
       </c>
-      <c r="I12" s="9" t="n">
+      <c r="I12" s="34" t="n">
         <v>6356</v>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -2378,13 +2398,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="33" t="n">
         <v>16018.5</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="33" t="n">
         <v>800.9299999999999</v>
       </c>
-      <c r="I13" s="5" t="n">
+      <c r="I13" s="33" t="n">
         <v>16819</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -2432,13 +2452,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" s="34" t="n">
         <v>38448</v>
       </c>
-      <c r="H14" s="9" t="n">
+      <c r="H14" s="34" t="n">
         <v>1922.42</v>
       </c>
-      <c r="I14" s="9" t="n">
+      <c r="I14" s="34" t="n">
         <v>40370</v>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -2486,13 +2506,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="33" t="n">
         <v>67615.32000000001</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="33" t="n">
         <v>3380.79</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="I15" s="33" t="n">
         <v>70996</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -2540,13 +2560,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G16" s="34" t="n">
         <v>26222.76</v>
       </c>
-      <c r="H16" s="9" t="n">
+      <c r="H16" s="34" t="n">
         <v>1311.15</v>
       </c>
-      <c r="I16" s="9" t="n">
+      <c r="I16" s="34" t="n">
         <v>27534</v>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -2594,13 +2614,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n">
+      <c r="G17" s="33" t="n">
         <v>148593.96</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="H17" s="33" t="n">
         <v>7429.7</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="I17" s="33" t="n">
         <v>156024</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -2648,13 +2668,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G18" s="9" t="n">
+      <c r="G18" s="34" t="n">
         <v>65895.84</v>
       </c>
-      <c r="H18" s="9" t="n">
+      <c r="H18" s="34" t="n">
         <v>3294.76</v>
       </c>
-      <c r="I18" s="9" t="n">
+      <c r="I18" s="34" t="n">
         <v>69191</v>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -2702,13 +2722,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G19" s="5" t="n">
+      <c r="G19" s="33" t="n">
         <v>51158.7</v>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="H19" s="33" t="n">
         <v>2557.94</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="I19" s="33" t="n">
         <v>53717</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -2756,13 +2776,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G20" s="9" t="n">
+      <c r="G20" s="34" t="n">
         <v>21136.74</v>
       </c>
-      <c r="H20" s="9" t="n">
+      <c r="H20" s="34" t="n">
         <v>1056.85</v>
       </c>
-      <c r="I20" s="9" t="n">
+      <c r="I20" s="34" t="n">
         <v>22194</v>
       </c>
       <c r="J20" s="8" t="inlineStr">
@@ -2810,13 +2830,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="G21" s="33" t="n">
         <v>32306.64</v>
       </c>
-      <c r="H21" s="5" t="n">
+      <c r="H21" s="33" t="n">
         <v>1615.33</v>
       </c>
-      <c r="I21" s="5" t="n">
+      <c r="I21" s="33" t="n">
         <v>33922</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2864,13 +2884,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G22" s="9" t="n">
+      <c r="G22" s="34" t="n">
         <v>14040</v>
       </c>
-      <c r="H22" s="9" t="n">
+      <c r="H22" s="34" t="n">
         <v>702</v>
       </c>
-      <c r="I22" s="9" t="n">
+      <c r="I22" s="34" t="n">
         <v>14742</v>
       </c>
       <c r="J22" s="8" t="inlineStr">
@@ -2918,13 +2938,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="G23" s="33" t="n">
         <v>71970.36</v>
       </c>
-      <c r="H23" s="5" t="n">
+      <c r="H23" s="33" t="n">
         <v>3598.53</v>
       </c>
-      <c r="I23" s="5" t="n">
+      <c r="I23" s="33" t="n">
         <v>75569</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2972,13 +2992,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G24" s="9" t="n">
+      <c r="G24" s="34" t="n">
         <v>33098.4</v>
       </c>
-      <c r="H24" s="9" t="n">
+      <c r="H24" s="34" t="n">
         <v>1654.92</v>
       </c>
-      <c r="I24" s="9" t="n">
+      <c r="I24" s="34" t="n">
         <v>34753</v>
       </c>
       <c r="J24" s="8" t="inlineStr">
@@ -3026,13 +3046,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="G25" s="33" t="n">
         <v>150038.88</v>
       </c>
-      <c r="H25" s="5" t="n">
+      <c r="H25" s="33" t="n">
         <v>7501.9</v>
       </c>
-      <c r="I25" s="5" t="n">
+      <c r="I25" s="33" t="n">
         <v>157541</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -3080,13 +3100,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G26" s="9" t="n">
+      <c r="G26" s="34" t="n">
         <v>14821.8</v>
       </c>
-      <c r="H26" s="9" t="n">
+      <c r="H26" s="34" t="n">
         <v>741.1</v>
       </c>
-      <c r="I26" s="9" t="n">
+      <c r="I26" s="34" t="n">
         <v>15563</v>
       </c>
       <c r="J26" s="8" t="inlineStr">
@@ -3134,13 +3154,13 @@
           <t>M/s Sushila Boot House, Jharsuguda</t>
         </is>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="G27" s="33" t="n">
         <v>162196.34</v>
       </c>
-      <c r="H27" s="5" t="n">
+      <c r="H27" s="33" t="n">
         <v>8109.79</v>
       </c>
-      <c r="I27" s="5" t="n">
+      <c r="I27" s="33" t="n">
         <v>170306</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -3188,13 +3208,13 @@
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G28" s="9" t="n">
+      <c r="G28" s="34" t="n">
         <v>21803.52</v>
       </c>
-      <c r="H28" s="9" t="n">
+      <c r="H28" s="34" t="n">
         <v>1090.16</v>
       </c>
-      <c r="I28" s="9" t="n">
+      <c r="I28" s="34" t="n">
         <v>22894</v>
       </c>
       <c r="J28" s="8" t="inlineStr">
@@ -3242,13 +3262,13 @@
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="G29" s="33" t="n">
         <v>17959.08</v>
       </c>
-      <c r="H29" s="5" t="n">
+      <c r="H29" s="33" t="n">
         <v>897.95</v>
       </c>
-      <c r="I29" s="5" t="n">
+      <c r="I29" s="33" t="n">
         <v>18857</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -3296,13 +3316,13 @@
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G30" s="9" t="n">
+      <c r="G30" s="34" t="n">
         <v>4036.2</v>
       </c>
-      <c r="H30" s="9" t="n">
+      <c r="H30" s="34" t="n">
         <v>201.81</v>
       </c>
-      <c r="I30" s="9" t="n">
+      <c r="I30" s="34" t="n">
         <v>4238</v>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -3350,13 +3370,13 @@
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G31" s="5" t="n">
+      <c r="G31" s="33" t="n">
         <v>50893.44</v>
       </c>
-      <c r="H31" s="5" t="n">
+      <c r="H31" s="33" t="n">
         <v>2544.64</v>
       </c>
-      <c r="I31" s="5" t="n">
+      <c r="I31" s="33" t="n">
         <v>53438</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -3404,13 +3424,13 @@
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G32" s="9" t="n">
+      <c r="G32" s="34" t="n">
         <v>54079.08</v>
       </c>
-      <c r="H32" s="9" t="n">
+      <c r="H32" s="34" t="n">
         <v>2703.93</v>
       </c>
-      <c r="I32" s="9" t="n">
+      <c r="I32" s="34" t="n">
         <v>56783</v>
       </c>
       <c r="J32" s="8" t="inlineStr">
@@ -3458,13 +3478,13 @@
           <t>K G N Footware, Parvathipuram</t>
         </is>
       </c>
-      <c r="G33" s="5" t="n">
+      <c r="G33" s="33" t="n">
         <v>32519.7</v>
       </c>
-      <c r="H33" s="5" t="n">
+      <c r="H33" s="33" t="n">
         <v>1626</v>
       </c>
-      <c r="I33" s="5" t="n">
+      <c r="I33" s="33" t="n">
         <v>34146</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -3512,13 +3532,13 @@
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G34" s="9" t="n">
+      <c r="G34" s="34" t="n">
         <v>4393.2</v>
       </c>
-      <c r="H34" s="9" t="n">
+      <c r="H34" s="34" t="n">
         <v>219.66</v>
       </c>
-      <c r="I34" s="9" t="n">
+      <c r="I34" s="34" t="n">
         <v>4613</v>
       </c>
       <c r="J34" s="8" t="inlineStr">
@@ -3566,13 +3586,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="33" t="n">
         <v>19989</v>
       </c>
-      <c r="H35" s="5" t="n">
+      <c r="H35" s="33" t="n">
         <v>999.45</v>
       </c>
-      <c r="I35" s="5" t="n">
+      <c r="I35" s="33" t="n">
         <v>20988</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3620,13 +3640,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G36" s="9" t="n">
+      <c r="G36" s="34" t="n">
         <v>11928.9</v>
       </c>
-      <c r="H36" s="9" t="n">
+      <c r="H36" s="34" t="n">
         <v>596.45</v>
       </c>
-      <c r="I36" s="9" t="n">
+      <c r="I36" s="34" t="n">
         <v>12525</v>
       </c>
       <c r="J36" s="8" t="inlineStr">
@@ -3674,13 +3694,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G37" s="5" t="n">
+      <c r="G37" s="33" t="n">
         <v>11876.1</v>
       </c>
-      <c r="H37" s="5" t="n">
+      <c r="H37" s="33" t="n">
         <v>593.8099999999999</v>
       </c>
-      <c r="I37" s="5" t="n">
+      <c r="I37" s="33" t="n">
         <v>12470</v>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3728,13 +3748,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G38" s="9" t="n">
+      <c r="G38" s="34" t="n">
         <v>5696.7</v>
       </c>
-      <c r="H38" s="9" t="n">
+      <c r="H38" s="34" t="n">
         <v>284.84</v>
       </c>
-      <c r="I38" s="9" t="n">
+      <c r="I38" s="34" t="n">
         <v>5982</v>
       </c>
       <c r="J38" s="8" t="inlineStr">
@@ -3782,13 +3802,13 @@
           <t>Mahavir Shoe House, Dhenkanal</t>
         </is>
       </c>
-      <c r="G39" s="5" t="n">
+      <c r="G39" s="33" t="n">
         <v>254563.8</v>
       </c>
-      <c r="H39" s="5" t="n">
+      <c r="H39" s="33" t="n">
         <v>12728.19</v>
       </c>
-      <c r="I39" s="5" t="n">
+      <c r="I39" s="33" t="n">
         <v>267292</v>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3836,13 +3856,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G40" s="9" t="n">
+      <c r="G40" s="34" t="n">
         <v>12386.16</v>
       </c>
-      <c r="H40" s="9" t="n">
+      <c r="H40" s="34" t="n">
         <v>619.3</v>
       </c>
-      <c r="I40" s="9" t="n">
+      <c r="I40" s="34" t="n">
         <v>13005</v>
       </c>
       <c r="J40" s="8" t="inlineStr">
@@ -3890,13 +3910,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G41" s="5" t="n">
+      <c r="G41" s="33" t="n">
         <v>22786.2</v>
       </c>
-      <c r="H41" s="5" t="n">
+      <c r="H41" s="33" t="n">
         <v>1139.32</v>
       </c>
-      <c r="I41" s="5" t="n">
+      <c r="I41" s="33" t="n">
         <v>23926</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3944,13 +3964,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G42" s="9" t="n">
+      <c r="G42" s="34" t="n">
         <v>9959.52</v>
       </c>
-      <c r="H42" s="9" t="n">
+      <c r="H42" s="34" t="n">
         <v>497.98</v>
       </c>
-      <c r="I42" s="9" t="n">
+      <c r="I42" s="34" t="n">
         <v>10458</v>
       </c>
       <c r="J42" s="8" t="inlineStr">
@@ -3998,13 +4018,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G43" s="5" t="n">
+      <c r="G43" s="33" t="n">
         <v>5339.4</v>
       </c>
-      <c r="H43" s="5" t="n">
+      <c r="H43" s="33" t="n">
         <v>266.97</v>
       </c>
-      <c r="I43" s="5" t="n">
+      <c r="I43" s="33" t="n">
         <v>5606</v>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -4052,13 +4072,13 @@
           <t>Sri Sharvani Traders, Visakhapatnam</t>
         </is>
       </c>
-      <c r="G44" s="9" t="n">
+      <c r="G44" s="34" t="n">
         <v>287637.24</v>
       </c>
-      <c r="H44" s="9" t="n">
+      <c r="H44" s="34" t="n">
         <v>14381.87</v>
       </c>
-      <c r="I44" s="9" t="n">
+      <c r="I44" s="34" t="n">
         <v>302019</v>
       </c>
       <c r="J44" s="8" t="inlineStr">
@@ -4106,13 +4126,13 @@
           <t>Jyothi Footwear, Vizianagaram</t>
         </is>
       </c>
-      <c r="G45" s="5" t="n">
+      <c r="G45" s="33" t="n">
         <v>74536.92</v>
       </c>
-      <c r="H45" s="5" t="n">
+      <c r="H45" s="33" t="n">
         <v>3726.85</v>
       </c>
-      <c r="I45" s="5" t="n">
+      <c r="I45" s="33" t="n">
         <v>78264</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -4160,13 +4180,13 @@
           <t>Sri Sharvani Traders, Visakhapatnam</t>
         </is>
       </c>
-      <c r="G46" s="9" t="n">
+      <c r="G46" s="34" t="n">
         <v>47888.16</v>
       </c>
-      <c r="H46" s="9" t="n">
+      <c r="H46" s="34" t="n">
         <v>2394.39</v>
       </c>
-      <c r="I46" s="9" t="n">
+      <c r="I46" s="34" t="n">
         <v>50283</v>
       </c>
       <c r="J46" s="8" t="inlineStr">
@@ -4214,13 +4234,13 @@
           <t>Sri Sharvani Traders, Visakhapatnam</t>
         </is>
       </c>
-      <c r="G47" s="5" t="n">
+      <c r="G47" s="33" t="n">
         <v>37721.64</v>
       </c>
-      <c r="H47" s="5" t="n">
+      <c r="H47" s="33" t="n">
         <v>1886.09</v>
       </c>
-      <c r="I47" s="5" t="n">
+      <c r="I47" s="33" t="n">
         <v>39608</v>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -4268,13 +4288,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G48" s="9" t="n">
+      <c r="G48" s="34" t="n">
         <v>36525.72</v>
       </c>
-      <c r="H48" s="9" t="n">
+      <c r="H48" s="34" t="n">
         <v>1826.27</v>
       </c>
-      <c r="I48" s="9" t="n">
+      <c r="I48" s="34" t="n">
         <v>38352</v>
       </c>
       <c r="J48" s="8" t="inlineStr">
@@ -4322,13 +4342,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G49" s="5" t="n">
+      <c r="G49" s="33" t="n">
         <v>23500.2</v>
       </c>
-      <c r="H49" s="5" t="n">
+      <c r="H49" s="33" t="n">
         <v>1175.02</v>
       </c>
-      <c r="I49" s="5" t="n">
+      <c r="I49" s="33" t="n">
         <v>24675</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -4376,13 +4396,13 @@
           <t>M/s Sri Brundabana Enterprises, Rayagada</t>
         </is>
       </c>
-      <c r="G50" s="9" t="n">
+      <c r="G50" s="34" t="n">
         <v>23139.18</v>
       </c>
-      <c r="H50" s="9" t="n">
+      <c r="H50" s="34" t="n">
         <v>1156.96</v>
       </c>
-      <c r="I50" s="9" t="n">
+      <c r="I50" s="34" t="n">
         <v>24296</v>
       </c>
       <c r="J50" s="8" t="inlineStr">
@@ -4430,13 +4450,13 @@
           <t>Sri Sharvani Traders, Visakhapatnam</t>
         </is>
       </c>
-      <c r="G51" s="5" t="n">
+      <c r="G51" s="33" t="n">
         <v>41721.6</v>
       </c>
-      <c r="H51" s="5" t="n">
+      <c r="H51" s="33" t="n">
         <v>2086.08</v>
       </c>
-      <c r="I51" s="5" t="n">
+      <c r="I51" s="33" t="n">
         <v>43808</v>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -4484,13 +4504,13 @@
           <t>M/s Sri Brundabana Enterprises, Malkangiri</t>
         </is>
       </c>
-      <c r="G52" s="9" t="n">
+      <c r="G52" s="34" t="n">
         <v>26716.8</v>
       </c>
-      <c r="H52" s="9" t="n">
+      <c r="H52" s="34" t="n">
         <v>1335.84</v>
       </c>
-      <c r="I52" s="9" t="n">
+      <c r="I52" s="34" t="n">
         <v>28053</v>
       </c>
       <c r="J52" s="8" t="inlineStr">
@@ -4538,13 +4558,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G53" s="5" t="n">
+      <c r="G53" s="33" t="n">
         <v>8283.120000000001</v>
       </c>
-      <c r="H53" s="5" t="n">
+      <c r="H53" s="33" t="n">
         <v>414.15</v>
       </c>
-      <c r="I53" s="5" t="n">
+      <c r="I53" s="33" t="n">
         <v>8697</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -4592,13 +4612,13 @@
           <t>M/s Sri Brundabana Enterprises, Malkangiri</t>
         </is>
       </c>
-      <c r="G54" s="9" t="n">
+      <c r="G54" s="34" t="n">
         <v>5696.7</v>
       </c>
-      <c r="H54" s="9" t="n">
+      <c r="H54" s="34" t="n">
         <v>284.84</v>
       </c>
-      <c r="I54" s="9" t="n">
+      <c r="I54" s="34" t="n">
         <v>5982</v>
       </c>
       <c r="J54" s="8" t="inlineStr">
@@ -4646,13 +4666,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G55" s="5" t="n">
+      <c r="G55" s="33" t="n">
         <v>14875.8</v>
       </c>
-      <c r="H55" s="5" t="n">
+      <c r="H55" s="33" t="n">
         <v>743.8</v>
       </c>
-      <c r="I55" s="5" t="n">
+      <c r="I55" s="33" t="n">
         <v>15620</v>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -4700,13 +4720,13 @@
           <t>M/s Sri Brundabana Enterprises, Malkangiri</t>
         </is>
       </c>
-      <c r="G56" s="9" t="n">
+      <c r="G56" s="34" t="n">
         <v>61896.78</v>
       </c>
-      <c r="H56" s="9" t="n">
+      <c r="H56" s="34" t="n">
         <v>3094.85</v>
       </c>
-      <c r="I56" s="9" t="n">
+      <c r="I56" s="34" t="n">
         <v>64992</v>
       </c>
       <c r="J56" s="8" t="inlineStr">
@@ -4754,13 +4774,13 @@
           <t>M/s. Shree Footwear, Srikakulam</t>
         </is>
       </c>
-      <c r="G57" s="5" t="n">
+      <c r="G57" s="33" t="n">
         <v>21536.7</v>
       </c>
-      <c r="H57" s="5" t="n">
+      <c r="H57" s="33" t="n">
         <v>1076.84</v>
       </c>
-      <c r="I57" s="5" t="n">
+      <c r="I57" s="33" t="n">
         <v>22614</v>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -4808,13 +4828,13 @@
           <t>Mahavir Shoe House, Dhenkanal</t>
         </is>
       </c>
-      <c r="G58" s="9" t="n">
+      <c r="G58" s="34" t="n">
         <v>134953.2</v>
       </c>
-      <c r="H58" s="9" t="n">
+      <c r="H58" s="34" t="n">
         <v>6747.66</v>
       </c>
-      <c r="I58" s="9" t="n">
+      <c r="I58" s="34" t="n">
         <v>141701</v>
       </c>
       <c r="J58" s="8" t="inlineStr">
@@ -4862,13 +4882,13 @@
           <t>SHREE ADITYA FOOT FASHION</t>
         </is>
       </c>
-      <c r="G59" s="5" t="n">
+      <c r="G59" s="33" t="n">
         <v>105402</v>
       </c>
-      <c r="H59" s="5" t="n">
+      <c r="H59" s="33" t="n">
         <v>5270.1</v>
       </c>
-      <c r="I59" s="5" t="n">
+      <c r="I59" s="33" t="n">
         <v>110672</v>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -4916,13 +4936,13 @@
           <t>M/S. RAJAN TRADERS</t>
         </is>
       </c>
-      <c r="G60" s="9" t="n">
+      <c r="G60" s="34" t="n">
         <v>104874</v>
       </c>
-      <c r="H60" s="9" t="n">
+      <c r="H60" s="34" t="n">
         <v>5243.7</v>
       </c>
-      <c r="I60" s="9" t="n">
+      <c r="I60" s="34" t="n">
         <v>110118</v>
       </c>
       <c r="J60" s="8" t="inlineStr">
@@ -4970,13 +4990,13 @@
           <t>SHREE ADITYA FOOT FASHION</t>
         </is>
       </c>
-      <c r="G61" s="5" t="n">
+      <c r="G61" s="33" t="n">
         <v>13752</v>
       </c>
-      <c r="H61" s="5" t="n">
+      <c r="H61" s="33" t="n">
         <v>687.6</v>
       </c>
-      <c r="I61" s="5" t="n">
+      <c r="I61" s="33" t="n">
         <v>14440</v>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -5010,13 +5030,13 @@
       <c r="D62" s="31" t="n"/>
       <c r="E62" s="31" t="n"/>
       <c r="F62" s="31" t="n"/>
-      <c r="G62" s="32" t="n">
+      <c r="G62" s="38" t="n">
         <v>2965194.44</v>
       </c>
-      <c r="H62" s="32" t="n">
+      <c r="H62" s="38" t="n">
         <v>148259.69</v>
       </c>
-      <c r="I62" s="32" t="n">
+      <c r="I62" s="38" t="n">
         <v>3113457.5</v>
       </c>
       <c r="J62" s="12" t="inlineStr">
@@ -5071,6 +5091,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="30" t="inlineStr">
         <is>
@@ -5144,13 +5165,13 @@
           <t>3.78% Retail Scheme (August 2026 Purchases)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="33" t="n">
         <v>43710.48</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="33" t="n">
         <v>2185.52</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="33" t="n">
         <v>45896</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -5190,13 +5211,13 @@
           <t>3.00% Cash Discount (August Prompt Settlement)</t>
         </is>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="34" t="n">
         <v>35763.92</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="F6" s="34" t="n">
         <v>1788.2</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="34" t="n">
         <v>37552.12</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -5236,13 +5257,13 @@
           <t>Rate Difference Rebate (UL 979E/CH+M Settlement)</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="33" t="n">
         <v>2641.86</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="33" t="n">
         <v>132.09</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="33" t="n">
         <v>2773.95</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -5282,13 +5303,13 @@
           <t>Non-Bengal Scratch Coupon Scheme (Aug Promo)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="34" t="n">
         <v>24501.9</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F8" s="34" t="n">
         <v>1225.1</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="34" t="n">
         <v>25727</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -5328,13 +5349,13 @@
           <t>2.00% QTB / Cash Discount (Sep 2026 Settlement)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="33" t="n">
         <v>19945.71</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="33" t="n">
         <v>997.29</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="33" t="n">
         <v>20943</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -5374,13 +5395,13 @@
           <t>Slab Scheme Bonus (Sep New State Target Bonus)</t>
         </is>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="34" t="n">
         <v>24933.33</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="34" t="n">
         <v>1246.67</v>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G10" s="34" t="n">
         <v>26180</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -5420,13 +5441,13 @@
           <t>3.78% Retail Scheme (September 2026 Purchases)</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="33" t="n">
         <v>37699.05</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="33" t="n">
         <v>1884.95</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="33" t="n">
         <v>39584</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -5458,13 +5479,13 @@
       </c>
       <c r="C12" s="31" t="n"/>
       <c r="D12" s="31" t="n"/>
-      <c r="E12" s="32" t="n">
+      <c r="E12" s="38" t="n">
         <v>189196.25</v>
       </c>
-      <c r="F12" s="32" t="n">
+      <c r="F12" s="38" t="n">
         <v>9459.82</v>
       </c>
-      <c r="G12" s="32" t="n">
+      <c r="G12" s="38" t="n">
         <v>198656.07</v>
       </c>
       <c r="H12" s="31" t="n"/>

</xml_diff>